<commit_message>
#36: batch-upload: added file attachments.
</commit_message>
<xml_diff>
--- a/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
+++ b/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/Shared Documents/Persistent ID for Instruments (PIDINST)/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Drive_D\projects\avre\apps\PIDINST\AuScope-instrument-registry\ckan_batch\src\ckan_batch\reader\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="281" documentId="13_ncr:1_{2C786F45-0395-42E9-BA7F-185CF1F6892D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{074526F3-620A-4F08-AC9F-C26815632F64}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6276FFB-5FF0-4D7F-88F0-6C513B3721F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="192">
   <si>
     <t>PIDINST Batch Instrument Upload Template (single-sheet, arrays via repeated rows)</t>
   </si>
@@ -584,6 +584,66 @@
   </si>
   <si>
     <t>Temperature,Conductivity</t>
+  </si>
+  <si>
+    <t>IsCover</t>
+  </si>
+  <si>
+    <t>Format</t>
+  </si>
+  <si>
+    <t>ATTACHMENTS</t>
+  </si>
+  <si>
+    <t>RESOURCES</t>
+  </si>
+  <si>
+    <t>local path to the file</t>
+  </si>
+  <si>
+    <t>The name of the resource (will be auto-generated from file name if not provided)</t>
+  </si>
+  <si>
+    <t>Is it the cover image</t>
+  </si>
+  <si>
+    <t>Format of the file: PDF | CSV | PNG, etc. (OPTIONAL)</t>
+  </si>
+  <si>
+    <t>Yes/No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Path</t>
+  </si>
+  <si>
+    <t>cover image</t>
+  </si>
+  <si>
+    <t>jpg</t>
+  </si>
+  <si>
+    <t>image</t>
+  </si>
+  <si>
+    <t>data</t>
+  </si>
+  <si>
+    <t>csv</t>
+  </si>
+  <si>
+    <t>~\CSIRO\AuScope AVRE - Persistent ID for Instruments (PIDINST)\data\accessories-for-mineralogy-microscopes.jpg</t>
+  </si>
+  <si>
+    <t>~\CSIRO\AuScope AVRE - Persistent ID for Instruments (PIDINST)\data\MDU-Hylogger-drill-core.jpg</t>
+  </si>
+  <si>
+    <t>~\Downloads\maia-statistics-2026-03-03T04-12-50.csv</t>
   </si>
 </sst>
 </file>
@@ -650,7 +710,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -708,8 +768,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -831,11 +903,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA6A6A6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFA6A6A6"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA6A6A6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -865,26 +957,23 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -905,6 +994,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -932,6 +1030,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1148,7 +1258,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AU5002"/>
+  <dimension ref="A1:AZ5002"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1192,123 +1302,142 @@
     <col min="45" max="45" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="10" customWidth="1"/>
+    <col min="48" max="48" width="46.28515625" customWidth="1"/>
+    <col min="49" max="49" width="22" customWidth="1"/>
+    <col min="50" max="50" width="12.140625" customWidth="1"/>
+    <col min="51" max="51" width="18.28515625" customWidth="1"/>
+    <col min="52" max="52" width="28.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:52" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="7"/>
     </row>
-    <row r="2" spans="1:47" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+    <row r="2" spans="1:52" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
-      <c r="X2" s="19"/>
-      <c r="Y2" s="19"/>
-      <c r="Z2" s="19"/>
-      <c r="AA2" s="19"/>
-      <c r="AB2" s="19"/>
-      <c r="AC2" s="19"/>
-      <c r="AD2" s="19"/>
-      <c r="AE2" s="19"/>
-      <c r="AF2" s="19"/>
-      <c r="AG2" s="19"/>
-      <c r="AH2" s="19"/>
-      <c r="AI2" s="20" t="s">
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
+      <c r="Q2" s="41"/>
+      <c r="R2" s="41"/>
+      <c r="S2" s="41"/>
+      <c r="T2" s="41"/>
+      <c r="U2" s="41"/>
+      <c r="V2" s="41"/>
+      <c r="W2" s="41"/>
+      <c r="X2" s="41"/>
+      <c r="Y2" s="41"/>
+      <c r="Z2" s="41"/>
+      <c r="AA2" s="41"/>
+      <c r="AB2" s="41"/>
+      <c r="AC2" s="41"/>
+      <c r="AD2" s="41"/>
+      <c r="AE2" s="41"/>
+      <c r="AF2" s="41"/>
+      <c r="AG2" s="41"/>
+      <c r="AH2" s="41"/>
+      <c r="AI2" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="AJ2" s="20"/>
-      <c r="AK2" s="20"/>
-      <c r="AL2" s="20"/>
-      <c r="AM2" s="20"/>
-      <c r="AN2" s="20"/>
-      <c r="AO2" s="20"/>
-      <c r="AP2" s="20"/>
-      <c r="AQ2" s="20"/>
-      <c r="AR2" s="20"/>
-      <c r="AS2" s="20"/>
-      <c r="AT2" s="20"/>
-      <c r="AU2" s="20"/>
-    </row>
-    <row r="3" spans="1:47" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AJ2" s="19"/>
+      <c r="AK2" s="19"/>
+      <c r="AL2" s="19"/>
+      <c r="AM2" s="19"/>
+      <c r="AN2" s="19"/>
+      <c r="AO2" s="19"/>
+      <c r="AP2" s="19"/>
+      <c r="AQ2" s="19"/>
+      <c r="AR2" s="19"/>
+      <c r="AS2" s="19"/>
+      <c r="AT2" s="19"/>
+      <c r="AU2" s="19"/>
+      <c r="AV2" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="AW2" s="19"/>
+      <c r="AX2" s="19"/>
+      <c r="AY2" s="19"/>
+      <c r="AZ2" s="19"/>
+    </row>
+    <row r="3" spans="1:52" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="12"/>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="23"/>
-      <c r="M3" s="30" t="s">
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="32" t="s">
         <v>163</v>
       </c>
-      <c r="N3" s="31"/>
-      <c r="O3" s="31"/>
-      <c r="P3" s="31"/>
-      <c r="Q3" s="31"/>
-      <c r="R3" s="31"/>
-      <c r="S3" s="31"/>
-      <c r="T3" s="31"/>
-      <c r="U3" s="31"/>
-      <c r="V3" s="31"/>
-      <c r="W3" s="31"/>
-      <c r="X3" s="31"/>
-      <c r="Y3" s="31"/>
-      <c r="Z3" s="31"/>
-      <c r="AA3" s="31"/>
-      <c r="AB3" s="31"/>
-      <c r="AC3" s="31"/>
-      <c r="AD3" s="31"/>
-      <c r="AE3" s="31"/>
-      <c r="AF3" s="31"/>
-      <c r="AG3" s="31"/>
-      <c r="AH3" s="32"/>
-      <c r="AI3" s="33" t="s">
+      <c r="N3" s="33"/>
+      <c r="O3" s="33"/>
+      <c r="P3" s="33"/>
+      <c r="Q3" s="33"/>
+      <c r="R3" s="33"/>
+      <c r="S3" s="33"/>
+      <c r="T3" s="33"/>
+      <c r="U3" s="33"/>
+      <c r="V3" s="33"/>
+      <c r="W3" s="33"/>
+      <c r="X3" s="33"/>
+      <c r="Y3" s="33"/>
+      <c r="Z3" s="33"/>
+      <c r="AA3" s="33"/>
+      <c r="AB3" s="33"/>
+      <c r="AC3" s="33"/>
+      <c r="AD3" s="33"/>
+      <c r="AE3" s="33"/>
+      <c r="AF3" s="33"/>
+      <c r="AG3" s="33"/>
+      <c r="AH3" s="34"/>
+      <c r="AI3" s="35" t="s">
         <v>164</v>
       </c>
-      <c r="AJ3" s="34"/>
-      <c r="AK3" s="34"/>
-      <c r="AL3" s="34"/>
-      <c r="AM3" s="34"/>
-      <c r="AN3" s="34"/>
-      <c r="AO3" s="34"/>
-      <c r="AP3" s="34"/>
-      <c r="AQ3" s="34"/>
-      <c r="AR3" s="34"/>
-      <c r="AS3" s="34"/>
-      <c r="AT3" s="34"/>
-      <c r="AU3" s="35"/>
-    </row>
-    <row r="4" spans="1:47" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AJ3" s="36"/>
+      <c r="AK3" s="36"/>
+      <c r="AL3" s="36"/>
+      <c r="AM3" s="36"/>
+      <c r="AN3" s="36"/>
+      <c r="AO3" s="36"/>
+      <c r="AP3" s="36"/>
+      <c r="AQ3" s="36"/>
+      <c r="AR3" s="36"/>
+      <c r="AS3" s="36"/>
+      <c r="AT3" s="36"/>
+      <c r="AU3" s="37"/>
+      <c r="AV3" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="AW3" s="18"/>
+      <c r="AX3" s="18"/>
+      <c r="AY3" s="18"/>
+      <c r="AZ3" s="18"/>
+    </row>
+    <row r="4" spans="1:52" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9"/>
       <c r="B4" s="9" t="s">
         <v>168</v>
@@ -1316,76 +1445,83 @@
       <c r="C4" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="E4" s="25"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="24" t="s">
+      <c r="E4" s="24"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="H4" s="25"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="24" t="s">
+      <c r="H4" s="24"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="K4" s="25"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="16" t="s">
+      <c r="K4" s="24"/>
+      <c r="L4" s="25"/>
+      <c r="M4" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="N4" s="17"/>
-      <c r="O4" s="17"/>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="18"/>
-      <c r="R4" s="16" t="s">
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="Q4" s="28"/>
+      <c r="R4" s="26" t="s">
         <v>144</v>
       </c>
-      <c r="S4" s="18"/>
-      <c r="T4" s="16" t="s">
+      <c r="S4" s="28"/>
+      <c r="T4" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="U4" s="17"/>
-      <c r="V4" s="18"/>
-      <c r="W4" s="13" t="s">
+      <c r="U4" s="27"/>
+      <c r="V4" s="28"/>
+      <c r="W4" s="38" t="s">
         <v>160</v>
       </c>
-      <c r="X4" s="14"/>
-      <c r="Y4" s="14"/>
-      <c r="Z4" s="14"/>
-      <c r="AA4" s="15"/>
-      <c r="AB4" s="16" t="s">
+      <c r="X4" s="39"/>
+      <c r="Y4" s="39"/>
+      <c r="Z4" s="39"/>
+      <c r="AA4" s="40"/>
+      <c r="AB4" s="26" t="s">
         <v>161</v>
       </c>
-      <c r="AC4" s="17"/>
-      <c r="AD4" s="17"/>
-      <c r="AE4" s="17"/>
-      <c r="AF4" s="18"/>
-      <c r="AG4" s="16" t="s">
+      <c r="AC4" s="27"/>
+      <c r="AD4" s="27"/>
+      <c r="AE4" s="27"/>
+      <c r="AF4" s="28"/>
+      <c r="AG4" s="26" t="s">
         <v>152</v>
       </c>
-      <c r="AH4" s="18"/>
-      <c r="AI4" s="27" t="s">
+      <c r="AH4" s="28"/>
+      <c r="AI4" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="AJ4" s="28"/>
-      <c r="AK4" s="28"/>
-      <c r="AL4" s="28"/>
-      <c r="AM4" s="28"/>
-      <c r="AN4" s="29"/>
-      <c r="AO4" s="27" t="s">
+      <c r="AJ4" s="30"/>
+      <c r="AK4" s="30"/>
+      <c r="AL4" s="30"/>
+      <c r="AM4" s="30"/>
+      <c r="AN4" s="31"/>
+      <c r="AO4" s="29" t="s">
         <v>152</v>
       </c>
-      <c r="AP4" s="28"/>
-      <c r="AQ4" s="29"/>
-      <c r="AR4" s="27" t="s">
+      <c r="AP4" s="30"/>
+      <c r="AQ4" s="31"/>
+      <c r="AR4" s="29" t="s">
         <v>153</v>
       </c>
-      <c r="AS4" s="28"/>
-      <c r="AT4" s="28"/>
-      <c r="AU4" s="29"/>
-    </row>
-    <row r="5" spans="1:47" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AS4" s="30"/>
+      <c r="AT4" s="30"/>
+      <c r="AU4" s="31"/>
+      <c r="AV4" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="AW4" s="16"/>
+      <c r="AX4" s="16"/>
+      <c r="AY4" s="16"/>
+      <c r="AZ4" s="16"/>
+    </row>
+    <row r="5" spans="1:52" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>131</v>
       </c>
@@ -1527,8 +1663,23 @@
       <c r="AU5" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="6" spans="1:47" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AV5" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="AW5" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="AX5" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="AY5" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="AZ5" s="13" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:52" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>129</v>
       </c>
@@ -1656,8 +1807,20 @@
       <c r="AU6" s="2" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AV6" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="AW6" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AX6" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="AY6" s="14" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="7" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1784,8 +1947,20 @@
       <c r="AU7">
         <v>4326</v>
       </c>
-    </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AV7" t="s">
+        <v>189</v>
+      </c>
+      <c r="AW7" t="s">
+        <v>184</v>
+      </c>
+      <c r="AX7" t="s">
+        <v>181</v>
+      </c>
+      <c r="AY7" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="8" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
@@ -1900,29 +2075,56 @@
       <c r="AU8" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AV8" t="s">
+        <v>190</v>
+      </c>
+      <c r="AW8" t="s">
+        <v>186</v>
+      </c>
+      <c r="AX8" t="s">
+        <v>182</v>
+      </c>
+      <c r="AY8" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="9" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>1</v>
+      </c>
       <c r="R9" s="3"/>
-    </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AV9" t="s">
+        <v>191</v>
+      </c>
+      <c r="AW9" t="s">
+        <v>187</v>
+      </c>
+      <c r="AX9" t="s">
+        <v>182</v>
+      </c>
+      <c r="AY9" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="10" spans="1:52" x14ac:dyDescent="0.25">
       <c r="R10" s="3"/>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:52" x14ac:dyDescent="0.25">
       <c r="R11" s="3"/>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:52" x14ac:dyDescent="0.25">
       <c r="R12" s="3"/>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:52" x14ac:dyDescent="0.25">
       <c r="R13" s="3"/>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:52" x14ac:dyDescent="0.25">
       <c r="R14" s="3"/>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:52" x14ac:dyDescent="0.25">
       <c r="R15" s="3"/>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:52" x14ac:dyDescent="0.25">
       <c r="R16" s="3"/>
     </row>
     <row r="17" spans="18:18" x14ac:dyDescent="0.25">
@@ -16884,12 +17086,14 @@
       <c r="R5002" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="T4:V4"/>
+  <mergeCells count="20">
     <mergeCell ref="W4:AA4"/>
     <mergeCell ref="AB4:AF4"/>
     <mergeCell ref="AG4:AH4"/>
     <mergeCell ref="A2:AH2"/>
+    <mergeCell ref="AV4:AZ4"/>
+    <mergeCell ref="AV3:AZ3"/>
+    <mergeCell ref="AV2:AZ2"/>
     <mergeCell ref="AI2:AU2"/>
     <mergeCell ref="C3:L3"/>
     <mergeCell ref="D4:F4"/>
@@ -16902,6 +17106,7 @@
     <mergeCell ref="M3:AH3"/>
     <mergeCell ref="AI3:AU3"/>
     <mergeCell ref="R4:S4"/>
+    <mergeCell ref="T4:V4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -16911,7 +17116,7 @@
   <legacyDrawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="9">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="10">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0EC81A5F-1FEC-43D6-BC95-EB808A23E26C}">
           <x14:formula1>
             <xm:f>_lists!$A$52:$A$54</xm:f>
@@ -16966,6 +17171,12 @@
           </x14:formula1>
           <xm:sqref>AK7:AK1048576</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B06767BB-3B31-45E1-A681-98128DFD18C8}">
+          <x14:formula1>
+            <xm:f>_lists!$A$74:$A$75</xm:f>
+          </x14:formula1>
+          <xm:sqref>AX7:AX1048576</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>
@@ -16974,7 +17185,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A71"/>
+  <dimension ref="A1:A75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -17282,8 +17493,24 @@
         <v>155</v>
       </c>
     </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" s="8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>182</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Aptos"&amp;12&amp;KFF0000 OFFICIAL&amp;1#_x000D_</oddHeader>
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;12&amp;KFF0000 OFFICIAL</oddFooter>
@@ -17319,6 +17546,22 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
+      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
+      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
+    </_dlc_DocIdUrl>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -17327,7 +17570,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -17377,7 +17620,7 @@
 </spe:Receivers>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C458252014B43B48B36D6FD06F31079C" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8411b2fcd13e9c262f801c2de01d8359">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9357ce84-a672-4584-8ddb-e5b553dfe263" xmlns:ns3="f66f598c-5a54-48fa-b12a-3e2e658c8d92" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7559adb2811d00dbbd5f4bbaad764c99" ns2:_="" ns3:_="">
     <xsd:import namespace="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
@@ -17639,23 +17882,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
-      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
-      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
-    </_dlc_DocIdUrl>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
+    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -17663,7 +17901,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
@@ -17671,7 +17909,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70706F67-F4D0-436B-9C39-1388BCD46E53}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17688,15 +17926,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
-    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
#69: selecting funder from facility list.
</commit_message>
<xml_diff>
--- a/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
+++ b/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Drive_D\projects\avre\apps\PIDINST\AuScope-instrument-registry\ckan_batch\src\ckan_batch\reader\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6276FFB-5FF0-4D7F-88F0-6C513B3721F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F66B738D-5257-4D12-97A2-CDA6D62B4EAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -568,9 +568,6 @@
     <t>Mandatory if Date is defined</t>
   </si>
   <si>
-    <t>auscope</t>
-  </si>
-  <si>
     <t>This is the ORGANISATION in the SITE where the instrument belongs to</t>
   </si>
   <si>
@@ -644,6 +641,9 @@
   </si>
   <si>
     <t>~\Downloads\maia-statistics-2026-03-03T04-12-50.csv</t>
+  </si>
+  <si>
+    <t>auscope-org</t>
   </si>
 </sst>
 </file>
@@ -963,6 +963,27 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -996,15 +1017,6 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1030,18 +1042,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1316,217 +1316,217 @@
       <c r="B1" s="7"/>
     </row>
     <row r="2" spans="1:52" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41"/>
-      <c r="S2" s="41"/>
-      <c r="T2" s="41"/>
-      <c r="U2" s="41"/>
-      <c r="V2" s="41"/>
-      <c r="W2" s="41"/>
-      <c r="X2" s="41"/>
-      <c r="Y2" s="41"/>
-      <c r="Z2" s="41"/>
-      <c r="AA2" s="41"/>
-      <c r="AB2" s="41"/>
-      <c r="AC2" s="41"/>
-      <c r="AD2" s="41"/>
-      <c r="AE2" s="41"/>
-      <c r="AF2" s="41"/>
-      <c r="AG2" s="41"/>
-      <c r="AH2" s="41"/>
-      <c r="AI2" s="19" t="s">
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="21"/>
+      <c r="T2" s="21"/>
+      <c r="U2" s="21"/>
+      <c r="V2" s="21"/>
+      <c r="W2" s="21"/>
+      <c r="X2" s="21"/>
+      <c r="Y2" s="21"/>
+      <c r="Z2" s="21"/>
+      <c r="AA2" s="21"/>
+      <c r="AB2" s="21"/>
+      <c r="AC2" s="21"/>
+      <c r="AD2" s="21"/>
+      <c r="AE2" s="21"/>
+      <c r="AF2" s="21"/>
+      <c r="AG2" s="21"/>
+      <c r="AH2" s="21"/>
+      <c r="AI2" s="26" t="s">
         <v>147</v>
       </c>
-      <c r="AJ2" s="19"/>
-      <c r="AK2" s="19"/>
-      <c r="AL2" s="19"/>
-      <c r="AM2" s="19"/>
-      <c r="AN2" s="19"/>
-      <c r="AO2" s="19"/>
-      <c r="AP2" s="19"/>
-      <c r="AQ2" s="19"/>
-      <c r="AR2" s="19"/>
-      <c r="AS2" s="19"/>
-      <c r="AT2" s="19"/>
-      <c r="AU2" s="19"/>
-      <c r="AV2" s="19" t="s">
-        <v>175</v>
-      </c>
-      <c r="AW2" s="19"/>
-      <c r="AX2" s="19"/>
-      <c r="AY2" s="19"/>
-      <c r="AZ2" s="19"/>
+      <c r="AJ2" s="26"/>
+      <c r="AK2" s="26"/>
+      <c r="AL2" s="26"/>
+      <c r="AM2" s="26"/>
+      <c r="AN2" s="26"/>
+      <c r="AO2" s="26"/>
+      <c r="AP2" s="26"/>
+      <c r="AQ2" s="26"/>
+      <c r="AR2" s="26"/>
+      <c r="AS2" s="26"/>
+      <c r="AT2" s="26"/>
+      <c r="AU2" s="26"/>
+      <c r="AV2" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="AW2" s="26"/>
+      <c r="AX2" s="26"/>
+      <c r="AY2" s="26"/>
+      <c r="AZ2" s="26"/>
     </row>
     <row r="3" spans="1:52" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="12"/>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="27" t="s">
         <v>159</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="32" t="s">
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="36" t="s">
         <v>163</v>
       </c>
-      <c r="N3" s="33"/>
-      <c r="O3" s="33"/>
-      <c r="P3" s="33"/>
-      <c r="Q3" s="33"/>
-      <c r="R3" s="33"/>
-      <c r="S3" s="33"/>
-      <c r="T3" s="33"/>
-      <c r="U3" s="33"/>
-      <c r="V3" s="33"/>
-      <c r="W3" s="33"/>
-      <c r="X3" s="33"/>
-      <c r="Y3" s="33"/>
-      <c r="Z3" s="33"/>
-      <c r="AA3" s="33"/>
-      <c r="AB3" s="33"/>
-      <c r="AC3" s="33"/>
-      <c r="AD3" s="33"/>
-      <c r="AE3" s="33"/>
-      <c r="AF3" s="33"/>
-      <c r="AG3" s="33"/>
-      <c r="AH3" s="34"/>
-      <c r="AI3" s="35" t="s">
+      <c r="N3" s="37"/>
+      <c r="O3" s="37"/>
+      <c r="P3" s="37"/>
+      <c r="Q3" s="37"/>
+      <c r="R3" s="37"/>
+      <c r="S3" s="37"/>
+      <c r="T3" s="37"/>
+      <c r="U3" s="37"/>
+      <c r="V3" s="37"/>
+      <c r="W3" s="37"/>
+      <c r="X3" s="37"/>
+      <c r="Y3" s="37"/>
+      <c r="Z3" s="37"/>
+      <c r="AA3" s="37"/>
+      <c r="AB3" s="37"/>
+      <c r="AC3" s="37"/>
+      <c r="AD3" s="37"/>
+      <c r="AE3" s="37"/>
+      <c r="AF3" s="37"/>
+      <c r="AG3" s="37"/>
+      <c r="AH3" s="38"/>
+      <c r="AI3" s="39" t="s">
         <v>164</v>
       </c>
-      <c r="AJ3" s="36"/>
-      <c r="AK3" s="36"/>
-      <c r="AL3" s="36"/>
-      <c r="AM3" s="36"/>
-      <c r="AN3" s="36"/>
-      <c r="AO3" s="36"/>
-      <c r="AP3" s="36"/>
-      <c r="AQ3" s="36"/>
-      <c r="AR3" s="36"/>
-      <c r="AS3" s="36"/>
-      <c r="AT3" s="36"/>
-      <c r="AU3" s="37"/>
-      <c r="AV3" s="17" t="s">
-        <v>175</v>
-      </c>
-      <c r="AW3" s="18"/>
-      <c r="AX3" s="18"/>
-      <c r="AY3" s="18"/>
-      <c r="AZ3" s="18"/>
+      <c r="AJ3" s="40"/>
+      <c r="AK3" s="40"/>
+      <c r="AL3" s="40"/>
+      <c r="AM3" s="40"/>
+      <c r="AN3" s="40"/>
+      <c r="AO3" s="40"/>
+      <c r="AP3" s="40"/>
+      <c r="AQ3" s="40"/>
+      <c r="AR3" s="40"/>
+      <c r="AS3" s="40"/>
+      <c r="AT3" s="40"/>
+      <c r="AU3" s="41"/>
+      <c r="AV3" s="24" t="s">
+        <v>174</v>
+      </c>
+      <c r="AW3" s="25"/>
+      <c r="AX3" s="25"/>
+      <c r="AY3" s="25"/>
+      <c r="AZ3" s="25"/>
     </row>
     <row r="4" spans="1:52" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9"/>
       <c r="B4" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="30" t="s">
         <v>140</v>
       </c>
-      <c r="E4" s="24"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="23" t="s">
+      <c r="E4" s="31"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="H4" s="24"/>
-      <c r="I4" s="25"/>
-      <c r="J4" s="23" t="s">
+      <c r="H4" s="31"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="30" t="s">
         <v>142</v>
       </c>
-      <c r="K4" s="24"/>
-      <c r="L4" s="25"/>
-      <c r="M4" s="26" t="s">
+      <c r="K4" s="31"/>
+      <c r="L4" s="32"/>
+      <c r="M4" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="28"/>
-      <c r="R4" s="26" t="s">
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="S4" s="28"/>
-      <c r="T4" s="26" t="s">
+      <c r="S4" s="20"/>
+      <c r="T4" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="U4" s="27"/>
-      <c r="V4" s="28"/>
-      <c r="W4" s="38" t="s">
+      <c r="U4" s="19"/>
+      <c r="V4" s="20"/>
+      <c r="W4" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="X4" s="39"/>
-      <c r="Y4" s="39"/>
-      <c r="Z4" s="39"/>
-      <c r="AA4" s="40"/>
-      <c r="AB4" s="26" t="s">
+      <c r="X4" s="16"/>
+      <c r="Y4" s="16"/>
+      <c r="Z4" s="16"/>
+      <c r="AA4" s="17"/>
+      <c r="AB4" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="AC4" s="27"/>
-      <c r="AD4" s="27"/>
-      <c r="AE4" s="27"/>
-      <c r="AF4" s="28"/>
-      <c r="AG4" s="26" t="s">
+      <c r="AC4" s="19"/>
+      <c r="AD4" s="19"/>
+      <c r="AE4" s="19"/>
+      <c r="AF4" s="20"/>
+      <c r="AG4" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="AH4" s="28"/>
-      <c r="AI4" s="29" t="s">
+      <c r="AH4" s="20"/>
+      <c r="AI4" s="33" t="s">
         <v>162</v>
       </c>
-      <c r="AJ4" s="30"/>
-      <c r="AK4" s="30"/>
-      <c r="AL4" s="30"/>
-      <c r="AM4" s="30"/>
-      <c r="AN4" s="31"/>
-      <c r="AO4" s="29" t="s">
+      <c r="AJ4" s="34"/>
+      <c r="AK4" s="34"/>
+      <c r="AL4" s="34"/>
+      <c r="AM4" s="34"/>
+      <c r="AN4" s="35"/>
+      <c r="AO4" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="AP4" s="30"/>
-      <c r="AQ4" s="31"/>
-      <c r="AR4" s="29" t="s">
+      <c r="AP4" s="34"/>
+      <c r="AQ4" s="35"/>
+      <c r="AR4" s="33" t="s">
         <v>153</v>
       </c>
-      <c r="AS4" s="30"/>
-      <c r="AT4" s="30"/>
-      <c r="AU4" s="31"/>
-      <c r="AV4" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="AW4" s="16"/>
-      <c r="AX4" s="16"/>
-      <c r="AY4" s="16"/>
-      <c r="AZ4" s="16"/>
+      <c r="AS4" s="34"/>
+      <c r="AT4" s="34"/>
+      <c r="AU4" s="35"/>
+      <c r="AV4" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="AW4" s="23"/>
+      <c r="AX4" s="23"/>
+      <c r="AY4" s="23"/>
+      <c r="AZ4" s="23"/>
     </row>
     <row r="5" spans="1:52" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>131</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>130</v>
@@ -1664,16 +1664,16 @@
         <v>22</v>
       </c>
       <c r="AV5" s="13" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AW5" s="13" t="s">
         <v>2</v>
       </c>
       <c r="AX5" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="AY5" s="13" t="s">
         <v>172</v>
-      </c>
-      <c r="AY5" s="13" t="s">
-        <v>173</v>
       </c>
       <c r="AZ5" s="13" t="s">
         <v>4</v>
@@ -1684,7 +1684,7 @@
         <v>129</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>27</v>
@@ -1767,7 +1767,7 @@
       <c r="AE6" s="2"/>
       <c r="AF6" s="2"/>
       <c r="AG6" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AH6" s="2" t="s">
         <v>39</v>
@@ -1808,16 +1808,16 @@
         <v>59</v>
       </c>
       <c r="AV6" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AW6" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="AW6" s="14" t="s">
+      <c r="AX6" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="AX6" s="14" t="s">
+      <c r="AY6" s="14" t="s">
         <v>178</v>
-      </c>
-      <c r="AY6" s="14" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="7" spans="1:52" x14ac:dyDescent="0.25">
@@ -1825,7 +1825,7 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>166</v>
+        <v>191</v>
       </c>
       <c r="C7" t="s">
         <v>63</v>
@@ -1903,7 +1903,7 @@
         <v>68</v>
       </c>
       <c r="AG7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AH7" t="s">
         <v>69</v>
@@ -1948,16 +1948,16 @@
         <v>4326</v>
       </c>
       <c r="AV7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AW7" t="s">
+        <v>183</v>
+      </c>
+      <c r="AX7" t="s">
+        <v>180</v>
+      </c>
+      <c r="AY7" t="s">
         <v>184</v>
-      </c>
-      <c r="AX7" t="s">
-        <v>181</v>
-      </c>
-      <c r="AY7" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="8" spans="1:52" x14ac:dyDescent="0.25">
@@ -2076,16 +2076,16 @@
         <v>68</v>
       </c>
       <c r="AV8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AW8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AX8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AY8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.25">
@@ -2094,16 +2094,16 @@
       </c>
       <c r="R9" s="3"/>
       <c r="AV9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AW9" t="s">
+        <v>186</v>
+      </c>
+      <c r="AX9" t="s">
+        <v>181</v>
+      </c>
+      <c r="AY9" t="s">
         <v>187</v>
-      </c>
-      <c r="AX9" t="s">
-        <v>182</v>
-      </c>
-      <c r="AY9" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:52" x14ac:dyDescent="0.25">
@@ -17087,6 +17087,10 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="M3:AH3"/>
+    <mergeCell ref="AI3:AU3"/>
+    <mergeCell ref="R4:S4"/>
+    <mergeCell ref="T4:V4"/>
     <mergeCell ref="W4:AA4"/>
     <mergeCell ref="AB4:AF4"/>
     <mergeCell ref="AG4:AH4"/>
@@ -17103,10 +17107,6 @@
     <mergeCell ref="AI4:AN4"/>
     <mergeCell ref="AO4:AQ4"/>
     <mergeCell ref="AR4:AU4"/>
-    <mergeCell ref="M3:AH3"/>
-    <mergeCell ref="AI3:AU3"/>
-    <mergeCell ref="R4:S4"/>
-    <mergeCell ref="T4:V4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -17495,17 +17495,17 @@
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -17546,81 +17546,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
-      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
-      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
-    </_dlc_DocIdUrl>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C458252014B43B48B36D6FD06F31079C" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8411b2fcd13e9c262f801c2de01d8359">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9357ce84-a672-4584-8ddb-e5b553dfe263" xmlns:ns3="f66f598c-5a54-48fa-b12a-3e2e658c8d92" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7559adb2811d00dbbd5f4bbaad764c99" ns2:_="" ns3:_="">
     <xsd:import namespace="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
@@ -17882,34 +17807,82 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
-    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
+      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
+      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
+    </_dlc_DocIdUrl>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70706F67-F4D0-436B-9C39-1388BCD46E53}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17926,4 +17899,31 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
+    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
#36: fix default org_owner.
</commit_message>
<xml_diff>
--- a/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
+++ b/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Drive_D\projects\avre\apps\PIDINST\AuScope-instrument-registry\ckan_batch\src\ckan_batch\reader\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E5E16E-2669-4000-AA41-E82984AC7F69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80B33212-09D7-496D-8490-6C10D8F6CD38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30840" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1002,33 +1002,6 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1065,6 +1038,12 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1082,6 +1061,27 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1346,118 +1346,118 @@
       </c>
     </row>
     <row r="2" spans="1:48" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="25"/>
-      <c r="P2" s="25"/>
-      <c r="Q2" s="25"/>
-      <c r="R2" s="25"/>
-      <c r="S2" s="25"/>
-      <c r="T2" s="25"/>
-      <c r="U2" s="25"/>
-      <c r="V2" s="25"/>
-      <c r="W2" s="25"/>
-      <c r="X2" s="25"/>
-      <c r="Y2" s="25"/>
-      <c r="Z2" s="25"/>
-      <c r="AA2" s="25"/>
-      <c r="AB2" s="25"/>
-      <c r="AC2" s="30" t="s">
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
+      <c r="S2" s="16"/>
+      <c r="T2" s="16"/>
+      <c r="U2" s="16"/>
+      <c r="V2" s="16"/>
+      <c r="W2" s="16"/>
+      <c r="X2" s="16"/>
+      <c r="Y2" s="16"/>
+      <c r="Z2" s="16"/>
+      <c r="AA2" s="16"/>
+      <c r="AB2" s="16"/>
+      <c r="AC2" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="AD2" s="30"/>
-      <c r="AE2" s="30"/>
-      <c r="AF2" s="30"/>
-      <c r="AG2" s="30"/>
-      <c r="AH2" s="30"/>
-      <c r="AI2" s="30"/>
-      <c r="AJ2" s="30"/>
-      <c r="AK2" s="30"/>
-      <c r="AL2" s="30"/>
-      <c r="AM2" s="30"/>
-      <c r="AN2" s="30"/>
-      <c r="AO2" s="30"/>
-      <c r="AP2" s="30"/>
-      <c r="AQ2" s="30"/>
-      <c r="AR2" s="30" t="s">
+      <c r="AD2" s="21"/>
+      <c r="AE2" s="21"/>
+      <c r="AF2" s="21"/>
+      <c r="AG2" s="21"/>
+      <c r="AH2" s="21"/>
+      <c r="AI2" s="21"/>
+      <c r="AJ2" s="21"/>
+      <c r="AK2" s="21"/>
+      <c r="AL2" s="21"/>
+      <c r="AM2" s="21"/>
+      <c r="AN2" s="21"/>
+      <c r="AO2" s="21"/>
+      <c r="AP2" s="21"/>
+      <c r="AQ2" s="21"/>
+      <c r="AR2" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="AS2" s="30"/>
-      <c r="AT2" s="30"/>
-      <c r="AU2" s="30"/>
-      <c r="AV2" s="30"/>
+      <c r="AS2" s="21"/>
+      <c r="AT2" s="21"/>
+      <c r="AU2" s="21"/>
+      <c r="AV2" s="21"/>
     </row>
     <row r="3" spans="1:48" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="40" t="s">
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="33" t="s">
         <v>138</v>
       </c>
-      <c r="L3" s="41"/>
-      <c r="M3" s="41"/>
-      <c r="N3" s="41"/>
-      <c r="O3" s="41"/>
-      <c r="P3" s="41"/>
-      <c r="Q3" s="41"/>
-      <c r="R3" s="41"/>
-      <c r="S3" s="41"/>
-      <c r="T3" s="41"/>
-      <c r="U3" s="41"/>
-      <c r="V3" s="41"/>
-      <c r="W3" s="41"/>
-      <c r="X3" s="41"/>
-      <c r="Y3" s="41"/>
-      <c r="Z3" s="41"/>
-      <c r="AA3" s="41"/>
-      <c r="AB3" s="42"/>
-      <c r="AC3" s="16" t="s">
+      <c r="L3" s="34"/>
+      <c r="M3" s="34"/>
+      <c r="N3" s="34"/>
+      <c r="O3" s="34"/>
+      <c r="P3" s="34"/>
+      <c r="Q3" s="34"/>
+      <c r="R3" s="34"/>
+      <c r="S3" s="34"/>
+      <c r="T3" s="34"/>
+      <c r="U3" s="34"/>
+      <c r="V3" s="34"/>
+      <c r="W3" s="34"/>
+      <c r="X3" s="34"/>
+      <c r="Y3" s="34"/>
+      <c r="Z3" s="34"/>
+      <c r="AA3" s="34"/>
+      <c r="AB3" s="35"/>
+      <c r="AC3" s="36" t="s">
         <v>139</v>
       </c>
-      <c r="AD3" s="17"/>
-      <c r="AE3" s="17"/>
-      <c r="AF3" s="17"/>
-      <c r="AG3" s="17"/>
-      <c r="AH3" s="17"/>
-      <c r="AI3" s="17"/>
-      <c r="AJ3" s="17"/>
-      <c r="AK3" s="17"/>
-      <c r="AL3" s="17"/>
-      <c r="AM3" s="17"/>
-      <c r="AN3" s="17"/>
-      <c r="AO3" s="17"/>
-      <c r="AP3" s="17"/>
-      <c r="AQ3" s="18"/>
-      <c r="AR3" s="28" t="s">
+      <c r="AD3" s="37"/>
+      <c r="AE3" s="37"/>
+      <c r="AF3" s="37"/>
+      <c r="AG3" s="37"/>
+      <c r="AH3" s="37"/>
+      <c r="AI3" s="37"/>
+      <c r="AJ3" s="37"/>
+      <c r="AK3" s="37"/>
+      <c r="AL3" s="37"/>
+      <c r="AM3" s="37"/>
+      <c r="AN3" s="37"/>
+      <c r="AO3" s="37"/>
+      <c r="AP3" s="37"/>
+      <c r="AQ3" s="38"/>
+      <c r="AR3" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="AS3" s="29"/>
-      <c r="AT3" s="29"/>
-      <c r="AU3" s="29"/>
-      <c r="AV3" s="29"/>
+      <c r="AS3" s="20"/>
+      <c r="AT3" s="20"/>
+      <c r="AU3" s="20"/>
+      <c r="AV3" s="20"/>
     </row>
     <row r="4" spans="1:48" s="8" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9"/>
@@ -1470,74 +1470,74 @@
       <c r="D4" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="E4" s="34" t="s">
+      <c r="E4" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="F4" s="35"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="34" t="s">
+      <c r="F4" s="26"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="I4" s="35"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="19" t="s">
+      <c r="I4" s="26"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="28" t="s">
         <v>121</v>
       </c>
-      <c r="L4" s="21"/>
-      <c r="M4" s="19" t="s">
+      <c r="L4" s="29"/>
+      <c r="M4" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="N4" s="20"/>
-      <c r="O4" s="19" t="s">
+      <c r="N4" s="39"/>
+      <c r="O4" s="28" t="s">
         <v>123</v>
       </c>
-      <c r="P4" s="21"/>
-      <c r="Q4" s="22" t="s">
+      <c r="P4" s="29"/>
+      <c r="Q4" s="40" t="s">
         <v>199</v>
       </c>
-      <c r="R4" s="23"/>
-      <c r="S4" s="23"/>
-      <c r="T4" s="23"/>
-      <c r="U4" s="24"/>
-      <c r="V4" s="19" t="s">
+      <c r="R4" s="41"/>
+      <c r="S4" s="41"/>
+      <c r="T4" s="41"/>
+      <c r="U4" s="42"/>
+      <c r="V4" s="28" t="s">
         <v>200</v>
       </c>
-      <c r="W4" s="21"/>
-      <c r="X4" s="21"/>
-      <c r="Y4" s="21"/>
-      <c r="Z4" s="19" t="s">
+      <c r="W4" s="29"/>
+      <c r="X4" s="29"/>
+      <c r="Y4" s="29"/>
+      <c r="Z4" s="28" t="s">
         <v>129</v>
       </c>
-      <c r="AA4" s="21"/>
-      <c r="AB4" s="20"/>
-      <c r="AC4" s="37" t="s">
+      <c r="AA4" s="29"/>
+      <c r="AB4" s="39"/>
+      <c r="AC4" s="30" t="s">
         <v>137</v>
       </c>
-      <c r="AD4" s="38"/>
-      <c r="AE4" s="38"/>
-      <c r="AF4" s="39"/>
-      <c r="AG4" s="37" t="s">
+      <c r="AD4" s="31"/>
+      <c r="AE4" s="31"/>
+      <c r="AF4" s="32"/>
+      <c r="AG4" s="30" t="s">
         <v>129</v>
       </c>
-      <c r="AH4" s="39"/>
-      <c r="AI4" s="37" t="s">
+      <c r="AH4" s="32"/>
+      <c r="AI4" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="AJ4" s="38"/>
-      <c r="AK4" s="38"/>
-      <c r="AL4" s="38"/>
-      <c r="AM4" s="38"/>
-      <c r="AN4" s="38"/>
-      <c r="AO4" s="38"/>
-      <c r="AP4" s="38"/>
-      <c r="AQ4" s="39"/>
-      <c r="AR4" s="26" t="s">
+      <c r="AJ4" s="31"/>
+      <c r="AK4" s="31"/>
+      <c r="AL4" s="31"/>
+      <c r="AM4" s="31"/>
+      <c r="AN4" s="31"/>
+      <c r="AO4" s="31"/>
+      <c r="AP4" s="31"/>
+      <c r="AQ4" s="32"/>
+      <c r="AR4" s="17" t="s">
         <v>143</v>
       </c>
-      <c r="AS4" s="27"/>
-      <c r="AT4" s="27"/>
-      <c r="AU4" s="27"/>
-      <c r="AV4" s="27"/>
+      <c r="AS4" s="18"/>
+      <c r="AT4" s="18"/>
+      <c r="AU4" s="18"/>
+      <c r="AV4" s="18"/>
     </row>
     <row r="5" spans="1:48" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -1899,7 +1899,7 @@
         <v>203</v>
       </c>
       <c r="Y7">
-        <v>10240</v>
+        <v>1</v>
       </c>
       <c r="Z7" t="s">
         <v>194</v>
@@ -17053,6 +17053,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="Q4:U4"/>
+    <mergeCell ref="V4:Y4"/>
+    <mergeCell ref="Z4:AB4"/>
     <mergeCell ref="A2:AB2"/>
     <mergeCell ref="AR4:AV4"/>
     <mergeCell ref="AR3:AV3"/>
@@ -17069,9 +17072,6 @@
     <mergeCell ref="AC3:AQ3"/>
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="O4:P4"/>
-    <mergeCell ref="Q4:U4"/>
-    <mergeCell ref="V4:Y4"/>
-    <mergeCell ref="Z4:AB4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -17549,30 +17549,55 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
-      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
-      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
-    </_dlc_DocIdUrl>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C458252014B43B48B36D6FD06F31079C" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8411b2fcd13e9c262f801c2de01d8359">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9357ce84-a672-4584-8ddb-e5b553dfe263" xmlns:ns3="f66f598c-5a54-48fa-b12a-3e2e658c8d92" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7559adb2811d00dbbd5f4bbaad764c99" ns2:_="" ns3:_="">
     <xsd:import namespace="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
@@ -17834,76 +17859,40 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
+      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
+      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
+    </_dlc_DocIdUrl>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
-    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70706F67-F4D0-436B-9C39-1388BCD46E53}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -17922,10 +17911,21 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
+    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
#36: adding support for platforms and Coverage dates
</commit_message>
<xml_diff>
--- a/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
+++ b/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Drive_D\projects\avre\apps\PIDINST\AuScope-instrument-registry\ckan_batch\src\ckan_batch\reader\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BD72907-7372-4868-9A8C-EFC328B6F7E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52509374-D1E4-456D-A4AD-9F2B923FCB43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instruments" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="205">
   <si>
     <t>PIDINST Batch Instrument Upload Template (single-sheet, arrays via repeated rows)</t>
   </si>
@@ -227,9 +227,6 @@
   </si>
   <si>
     <t>ROR</t>
-  </si>
-  <si>
-    <t>SN-000099</t>
   </si>
   <si>
     <t>SerialNumber</t>
@@ -679,7 +676,13 @@
     <t>MTU-5C</t>
   </si>
   <si>
-    <t>Relevant date in YYYY or YYYY-MM or YYYY-MM-DD</t>
+    <t>SN-111111</t>
+  </si>
+  <si>
+    <t>Relevant date in YYYY or YYYY-MM or YYYY-MM-DD. For Coverage, you can provide range dates according to RKMS-ISO8601</t>
+  </si>
+  <si>
+    <t>Period of Activity</t>
   </si>
 </sst>
 </file>
@@ -960,7 +963,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -998,93 +1001,90 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1313,7 +1313,7 @@
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="11" width="22" customWidth="1"/>
     <col min="12" max="12" width="24" customWidth="1"/>
-    <col min="13" max="13" width="17.7109375" style="42" customWidth="1"/>
+    <col min="13" max="13" width="39.7109375" style="15" customWidth="1"/>
     <col min="14" max="14" width="22" customWidth="1"/>
     <col min="15" max="15" width="21.85546875" customWidth="1"/>
     <col min="16" max="16" width="27.42578125" bestFit="1" customWidth="1"/>
@@ -1349,280 +1349,280 @@
       </c>
     </row>
     <row r="2" spans="1:48" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="T2" s="17"/>
+      <c r="U2" s="17"/>
+      <c r="V2" s="17"/>
+      <c r="W2" s="17"/>
+      <c r="X2" s="17"/>
+      <c r="Y2" s="17"/>
+      <c r="Z2" s="17"/>
+      <c r="AA2" s="17"/>
+      <c r="AB2" s="17"/>
+      <c r="AC2" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="24"/>
-      <c r="P2" s="24"/>
-      <c r="Q2" s="24"/>
-      <c r="R2" s="24"/>
-      <c r="S2" s="24"/>
-      <c r="T2" s="24"/>
-      <c r="U2" s="24"/>
-      <c r="V2" s="24"/>
-      <c r="W2" s="24"/>
-      <c r="X2" s="24"/>
-      <c r="Y2" s="24"/>
-      <c r="Z2" s="24"/>
-      <c r="AA2" s="24"/>
-      <c r="AB2" s="24"/>
-      <c r="AC2" s="29" t="s">
-        <v>124</v>
-      </c>
-      <c r="AD2" s="29"/>
-      <c r="AE2" s="29"/>
-      <c r="AF2" s="29"/>
-      <c r="AG2" s="29"/>
-      <c r="AH2" s="29"/>
-      <c r="AI2" s="29"/>
-      <c r="AJ2" s="29"/>
-      <c r="AK2" s="29"/>
-      <c r="AL2" s="29"/>
-      <c r="AM2" s="29"/>
-      <c r="AN2" s="29"/>
-      <c r="AO2" s="29"/>
-      <c r="AP2" s="29"/>
-      <c r="AQ2" s="29"/>
-      <c r="AR2" s="29" t="s">
-        <v>143</v>
-      </c>
-      <c r="AS2" s="29"/>
-      <c r="AT2" s="29"/>
-      <c r="AU2" s="29"/>
-      <c r="AV2" s="29"/>
+      <c r="AD2" s="22"/>
+      <c r="AE2" s="22"/>
+      <c r="AF2" s="22"/>
+      <c r="AG2" s="22"/>
+      <c r="AH2" s="22"/>
+      <c r="AI2" s="22"/>
+      <c r="AJ2" s="22"/>
+      <c r="AK2" s="22"/>
+      <c r="AL2" s="22"/>
+      <c r="AM2" s="22"/>
+      <c r="AN2" s="22"/>
+      <c r="AO2" s="22"/>
+      <c r="AP2" s="22"/>
+      <c r="AQ2" s="22"/>
+      <c r="AR2" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="AS2" s="22"/>
+      <c r="AT2" s="22"/>
+      <c r="AU2" s="22"/>
+      <c r="AV2" s="22"/>
     </row>
     <row r="3" spans="1:48" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
-      <c r="B3" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="39" t="s">
+      <c r="B3" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
+      <c r="N3" s="35"/>
+      <c r="O3" s="35"/>
+      <c r="P3" s="35"/>
+      <c r="Q3" s="35"/>
+      <c r="R3" s="35"/>
+      <c r="S3" s="35"/>
+      <c r="T3" s="35"/>
+      <c r="U3" s="35"/>
+      <c r="V3" s="35"/>
+      <c r="W3" s="35"/>
+      <c r="X3" s="35"/>
+      <c r="Y3" s="35"/>
+      <c r="Z3" s="35"/>
+      <c r="AA3" s="35"/>
+      <c r="AB3" s="36"/>
+      <c r="AC3" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="40"/>
-      <c r="O3" s="40"/>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="40"/>
-      <c r="R3" s="40"/>
-      <c r="S3" s="40"/>
-      <c r="T3" s="40"/>
-      <c r="U3" s="40"/>
-      <c r="V3" s="40"/>
-      <c r="W3" s="40"/>
-      <c r="X3" s="40"/>
-      <c r="Y3" s="40"/>
-      <c r="Z3" s="40"/>
-      <c r="AA3" s="40"/>
-      <c r="AB3" s="41"/>
-      <c r="AC3" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="AD3" s="16"/>
-      <c r="AE3" s="16"/>
-      <c r="AF3" s="16"/>
-      <c r="AG3" s="16"/>
-      <c r="AH3" s="16"/>
-      <c r="AI3" s="16"/>
-      <c r="AJ3" s="16"/>
-      <c r="AK3" s="16"/>
-      <c r="AL3" s="16"/>
-      <c r="AM3" s="16"/>
-      <c r="AN3" s="16"/>
-      <c r="AO3" s="16"/>
-      <c r="AP3" s="16"/>
-      <c r="AQ3" s="17"/>
-      <c r="AR3" s="27" t="s">
-        <v>143</v>
-      </c>
-      <c r="AS3" s="28"/>
-      <c r="AT3" s="28"/>
-      <c r="AU3" s="28"/>
-      <c r="AV3" s="28"/>
+      <c r="AD3" s="38"/>
+      <c r="AE3" s="38"/>
+      <c r="AF3" s="38"/>
+      <c r="AG3" s="38"/>
+      <c r="AH3" s="38"/>
+      <c r="AI3" s="38"/>
+      <c r="AJ3" s="38"/>
+      <c r="AK3" s="38"/>
+      <c r="AL3" s="38"/>
+      <c r="AM3" s="38"/>
+      <c r="AN3" s="38"/>
+      <c r="AO3" s="38"/>
+      <c r="AP3" s="38"/>
+      <c r="AQ3" s="39"/>
+      <c r="AR3" s="20" t="s">
+        <v>142</v>
+      </c>
+      <c r="AS3" s="21"/>
+      <c r="AT3" s="21"/>
+      <c r="AU3" s="21"/>
+      <c r="AV3" s="21"/>
     </row>
     <row r="4" spans="1:48" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="C4" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="D4" s="13" t="s">
+      <c r="E4" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="F4" s="27"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="F4" s="34"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="33" t="s">
+      <c r="I4" s="27"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="29" t="s">
         <v>119</v>
       </c>
-      <c r="I4" s="34"/>
-      <c r="J4" s="35"/>
-      <c r="K4" s="18" t="s">
+      <c r="L4" s="30"/>
+      <c r="M4" s="29" t="s">
         <v>120</v>
       </c>
-      <c r="L4" s="20"/>
-      <c r="M4" s="18" t="s">
+      <c r="N4" s="40"/>
+      <c r="O4" s="29" t="s">
         <v>121</v>
       </c>
-      <c r="N4" s="19"/>
-      <c r="O4" s="18" t="s">
-        <v>122</v>
-      </c>
-      <c r="P4" s="20"/>
-      <c r="Q4" s="21" t="s">
+      <c r="P4" s="30"/>
+      <c r="Q4" s="41" t="s">
+        <v>197</v>
+      </c>
+      <c r="R4" s="42"/>
+      <c r="S4" s="42"/>
+      <c r="T4" s="42"/>
+      <c r="U4" s="43"/>
+      <c r="V4" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="R4" s="22"/>
-      <c r="S4" s="22"/>
-      <c r="T4" s="22"/>
-      <c r="U4" s="23"/>
-      <c r="V4" s="18" t="s">
-        <v>199</v>
-      </c>
-      <c r="W4" s="20"/>
-      <c r="X4" s="20"/>
-      <c r="Y4" s="20"/>
-      <c r="Z4" s="18" t="s">
+      <c r="W4" s="30"/>
+      <c r="X4" s="30"/>
+      <c r="Y4" s="30"/>
+      <c r="Z4" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA4" s="30"/>
+      <c r="AB4" s="40"/>
+      <c r="AC4" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="AD4" s="32"/>
+      <c r="AE4" s="32"/>
+      <c r="AF4" s="33"/>
+      <c r="AG4" s="31" t="s">
+        <v>127</v>
+      </c>
+      <c r="AH4" s="33"/>
+      <c r="AI4" s="31" t="s">
         <v>128</v>
       </c>
-      <c r="AA4" s="20"/>
-      <c r="AB4" s="19"/>
-      <c r="AC4" s="36" t="s">
-        <v>136</v>
-      </c>
-      <c r="AD4" s="37"/>
-      <c r="AE4" s="37"/>
-      <c r="AF4" s="38"/>
-      <c r="AG4" s="36" t="s">
-        <v>128</v>
-      </c>
-      <c r="AH4" s="38"/>
-      <c r="AI4" s="36" t="s">
-        <v>129</v>
-      </c>
-      <c r="AJ4" s="37"/>
-      <c r="AK4" s="37"/>
-      <c r="AL4" s="37"/>
-      <c r="AM4" s="37"/>
-      <c r="AN4" s="37"/>
-      <c r="AO4" s="37"/>
-      <c r="AP4" s="37"/>
-      <c r="AQ4" s="38"/>
-      <c r="AR4" s="25" t="s">
-        <v>142</v>
-      </c>
-      <c r="AS4" s="26"/>
-      <c r="AT4" s="26"/>
-      <c r="AU4" s="26"/>
-      <c r="AV4" s="26"/>
+      <c r="AJ4" s="32"/>
+      <c r="AK4" s="32"/>
+      <c r="AL4" s="32"/>
+      <c r="AM4" s="32"/>
+      <c r="AN4" s="32"/>
+      <c r="AO4" s="32"/>
+      <c r="AP4" s="32"/>
+      <c r="AQ4" s="33"/>
+      <c r="AR4" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="AS4" s="19"/>
+      <c r="AT4" s="19"/>
+      <c r="AU4" s="19"/>
+      <c r="AV4" s="19"/>
     </row>
     <row r="5" spans="1:48" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H5" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>134</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>2</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="M5" s="43" t="s">
+        <v>109</v>
+      </c>
+      <c r="M5" s="16" t="s">
         <v>5</v>
       </c>
       <c r="N5" s="10" t="s">
         <v>6</v>
       </c>
       <c r="O5" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="P5" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="P5" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="Q5" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="R5" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="R5" s="10" t="s">
-        <v>115</v>
-      </c>
       <c r="S5" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="T5" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="U5" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="T5" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="U5" s="10" t="s">
-        <v>126</v>
-      </c>
       <c r="V5" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="W5" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="X5" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="X5" s="10" t="s">
-        <v>113</v>
-      </c>
       <c r="Y5" s="10" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="Z5" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="AA5" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="AA5" s="1" t="s">
-        <v>166</v>
       </c>
       <c r="AB5" s="1" t="s">
         <v>4</v>
@@ -1649,40 +1649,40 @@
         <v>17</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AK5" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AL5" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AL5" s="1" t="s">
-        <v>106</v>
-      </c>
       <c r="AM5" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="AN5" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="AN5" s="1" t="s">
+      <c r="AO5" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="AO5" s="1" t="s">
+      <c r="AP5" s="1" t="s">
         <v>188</v>
-      </c>
-      <c r="AP5" s="1" t="s">
-        <v>189</v>
       </c>
       <c r="AQ5" s="1" t="s">
         <v>19</v>
       </c>
       <c r="AR5" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AS5" s="11" t="s">
         <v>2</v>
       </c>
       <c r="AT5" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="AU5" s="11" t="s">
         <v>140</v>
-      </c>
-      <c r="AU5" s="11" t="s">
-        <v>141</v>
       </c>
       <c r="AV5" s="11" t="s">
         <v>4</v>
@@ -1690,13 +1690,13 @@
     </row>
     <row r="6" spans="1:48" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>26</v>
@@ -1725,17 +1725,17 @@
       <c r="L6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="44" t="s">
+      <c r="M6" s="2" t="s">
         <v>203</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="O6" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="P6" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="P6" s="2" t="s">
-        <v>164</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>38</v>
@@ -1753,22 +1753,22 @@
         <v>42</v>
       </c>
       <c r="V6" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="W6" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="W6" s="2" t="s">
+      <c r="X6" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="X6" s="2" t="s">
-        <v>197</v>
-      </c>
       <c r="Y6" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Z6" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="AA6" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="AA6" s="2" t="s">
-        <v>168</v>
       </c>
       <c r="AB6" s="2" t="s">
         <v>30</v>
@@ -1795,40 +1795,40 @@
         <v>43</v>
       </c>
       <c r="AJ6" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AK6" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="AL6" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM6" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="AL6" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="AM6" s="2" t="s">
+      <c r="AN6" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AN6" s="2" t="s">
+      <c r="AO6" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AO6" s="2" t="s">
+      <c r="AP6" s="2" t="s">
         <v>179</v>
-      </c>
-      <c r="AP6" s="2" t="s">
-        <v>180</v>
       </c>
       <c r="AQ6" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AR6" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="AS6" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="AS6" s="12" t="s">
+      <c r="AT6" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="AT6" s="12" t="s">
+      <c r="AU6" s="12" t="s">
         <v>146</v>
-      </c>
-      <c r="AU6" s="12" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:48" x14ac:dyDescent="0.25">
@@ -1839,82 +1839,82 @@
         <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D7" t="s">
+        <v>189</v>
+      </c>
+      <c r="E7" t="s">
+        <v>131</v>
+      </c>
+      <c r="F7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" t="s">
+        <v>202</v>
+      </c>
+      <c r="I7" t="s">
+        <v>55</v>
+      </c>
+      <c r="J7" t="s">
+        <v>50</v>
+      </c>
+      <c r="K7" t="s">
         <v>190</v>
-      </c>
-      <c r="E7" t="s">
-        <v>132</v>
-      </c>
-      <c r="F7" t="s">
-        <v>50</v>
-      </c>
-      <c r="G7" t="s">
-        <v>50</v>
-      </c>
-      <c r="H7" t="s">
-        <v>55</v>
-      </c>
-      <c r="I7" t="s">
-        <v>56</v>
-      </c>
-      <c r="J7" t="s">
-        <v>50</v>
-      </c>
-      <c r="K7" t="s">
-        <v>191</v>
       </c>
       <c r="L7" t="s">
         <v>48</v>
       </c>
-      <c r="M7" s="42" t="s">
+      <c r="M7" s="15" t="s">
         <v>52</v>
       </c>
       <c r="N7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="O7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="P7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="Q7" t="s">
+        <v>56</v>
+      </c>
+      <c r="R7" t="s">
         <v>57</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>58</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>59</v>
       </c>
-      <c r="T7" t="s">
-        <v>60</v>
-      </c>
       <c r="U7" t="s">
         <v>50</v>
       </c>
       <c r="W7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="X7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Y7">
         <v>1</v>
       </c>
       <c r="Z7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AA7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AB7" t="s">
         <v>51</v>
       </c>
       <c r="AC7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AD7" t="s">
         <v>50</v>
@@ -1926,16 +1926,16 @@
         <v>50</v>
       </c>
       <c r="AG7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AH7" t="s">
         <v>50</v>
       </c>
       <c r="AI7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AJ7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AK7">
         <v>115.86</v>
@@ -1947,16 +1947,16 @@
         <v>4326</v>
       </c>
       <c r="AR7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AS7" t="s">
+        <v>151</v>
+      </c>
+      <c r="AT7" t="s">
+        <v>148</v>
+      </c>
+      <c r="AU7" t="s">
         <v>152</v>
-      </c>
-      <c r="AT7" t="s">
-        <v>149</v>
-      </c>
-      <c r="AU7" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:48" x14ac:dyDescent="0.25">
@@ -1979,10 +1979,10 @@
         <v>50</v>
       </c>
       <c r="H8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K8" t="s">
         <v>50</v>
@@ -1990,7 +1990,7 @@
       <c r="L8" t="s">
         <v>50</v>
       </c>
-      <c r="M8" s="42" t="s">
+      <c r="M8" s="15" t="s">
         <v>50</v>
       </c>
       <c r="N8" t="s">
@@ -2045,16 +2045,16 @@
         <v>50</v>
       </c>
       <c r="AR8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AS8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AT8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AU8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:48" x14ac:dyDescent="0.25">
@@ -2062,20 +2062,23 @@
         <v>1</v>
       </c>
       <c r="AR9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AS9" t="s">
+        <v>154</v>
+      </c>
+      <c r="AT9" t="s">
+        <v>149</v>
+      </c>
+      <c r="AU9" t="s">
         <v>155</v>
-      </c>
-      <c r="AT9" t="s">
-        <v>150</v>
-      </c>
-      <c r="AU9" t="s">
-        <v>156</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="Q4:U4"/>
+    <mergeCell ref="V4:Y4"/>
+    <mergeCell ref="Z4:AB4"/>
     <mergeCell ref="A2:AB2"/>
     <mergeCell ref="AR4:AV4"/>
     <mergeCell ref="AR3:AV3"/>
@@ -2092,9 +2095,6 @@
     <mergeCell ref="AC3:AQ3"/>
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="O4:P4"/>
-    <mergeCell ref="Q4:U4"/>
-    <mergeCell ref="V4:Y4"/>
-    <mergeCell ref="Z4:AB4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -2110,12 +2110,6 @@
             <xm:f>_lists!$A$52:$A$54</xm:f>
           </x14:formula1>
           <xm:sqref>I7:I1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A7C010E6-A2C8-4249-A233-D7E02A1F145B}">
-          <x14:formula1>
-            <xm:f>_lists!$A$70:$A$71</xm:f>
-          </x14:formula1>
-          <xm:sqref>N7:N1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D8B9F839-0BDE-4FD4-B802-1C94BF58BC01}">
           <x14:formula1>
@@ -2143,21 +2137,27 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B06767BB-3B31-45E1-A681-98128DFD18C8}">
           <x14:formula1>
-            <xm:f>_lists!$A$74:$A$75</xm:f>
+            <xm:f>_lists!$A$75:$A$76</xm:f>
           </x14:formula1>
           <xm:sqref>AT7:AT1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{92A0783E-8438-44B7-8D64-4FE7175FA9FB}">
           <x14:formula1>
-            <xm:f>_lists!$A$78:$A$80</xm:f>
+            <xm:f>_lists!$A$79:$A$81</xm:f>
           </x14:formula1>
           <xm:sqref>C7:C1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8E91E68E-1DCC-47C2-8753-4026B09E5314}">
           <x14:formula1>
-            <xm:f>_lists!$A$83:$A$85</xm:f>
+            <xm:f>_lists!$A$84:$A$86</xm:f>
           </x14:formula1>
           <xm:sqref>AJ7:AJ1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{56BC94EC-09BC-4572-B5EA-F8DA94792981}">
+          <x14:formula1>
+            <xm:f>_lists!$A$70:$A$72</xm:f>
+          </x14:formula1>
+          <xm:sqref>N7:N1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2167,7 +2167,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A85"/>
+  <dimension ref="A1:A86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" customWidth="1"/>
@@ -2185,12 +2185,12 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
@@ -2205,22 +2205,22 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -2230,87 +2230,87 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
@@ -2320,12 +2320,12 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
@@ -2335,22 +2335,22 @@
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
@@ -2360,37 +2360,37 @@
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
@@ -2400,17 +2400,17 @@
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
@@ -2420,12 +2420,12 @@
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
@@ -2435,12 +2435,12 @@
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
@@ -2455,12 +2455,12 @@
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
@@ -2470,67 +2470,72 @@
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" s="7" t="s">
-        <v>148</v>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>149</v>
+      <c r="A74" s="7" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" s="7" t="s">
-        <v>173</v>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+      <c r="A78" s="7" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82" s="7" t="s">
-        <v>183</v>
+        <v>173</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>99</v>
+      <c r="A83" s="7" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>184</v>
+        <v>98</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>100</v>
+        <v>183</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2553,12 +2558,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -2571,56 +2576,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C458252014B43B48B36D6FD06F31079C" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8411b2fcd13e9c262f801c2de01d8359">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9357ce84-a672-4584-8ddb-e5b553dfe263" xmlns:ns3="f66f598c-5a54-48fa-b12a-3e2e658c8d92" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7559adb2811d00dbbd5f4bbaad764c99" ns2:_="" ns3:_="">
     <xsd:import namespace="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
@@ -2882,7 +2837,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
@@ -2898,7 +2853,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2907,15 +2862,57 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70706F67-F4D0-436B-9C39-1388BCD46E53}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2934,7 +2931,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2945,10 +2942,18 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
#91: client_batch: adding batch update. adding export. prepared template notebooks for create and update.
</commit_message>
<xml_diff>
--- a/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
+++ b/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Drive_D\projects\avre\apps\PIDINST\AuScope-instrument-registry\ckan_batch\src\ckan_batch\reader\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52509374-D1E4-456D-A4AD-9F2B923FCB43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B29D50-AA81-4EFD-92E0-799103CE51F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30840" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instruments" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="README" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Instruments!$A$5:$AH$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Instruments!$A$5:$AI$5</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -32,7 +32,7 @@
     <author>tc={785D315C-EB53-42A1-A495-EF7EA88212BE}</author>
   </authors>
   <commentList>
-    <comment ref="O4" authorId="0" shapeId="0" xr:uid="{3449D359-B9EE-4FE3-8BA1-8E90EA1E9711}">
+    <comment ref="P4" authorId="0" shapeId="0" xr:uid="{3449D359-B9EE-4FE3-8BA1-8E90EA1E9711}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -40,7 +40,7 @@
     The first record on instrument type will also be picked for resourceType. This is just for mapping to DataCite</t>
       </text>
     </comment>
-    <comment ref="Q4" authorId="1" shapeId="0" xr:uid="{EB2AA444-AB45-471F-B2D2-3762B9440EA1}">
+    <comment ref="R4" authorId="1" shapeId="0" xr:uid="{EB2AA444-AB45-471F-B2D2-3762B9440EA1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -48,7 +48,7 @@
     Use this block for resources that are not registered in our Instrument Registry (e.g. related documents or datasets)</t>
       </text>
     </comment>
-    <comment ref="V4" authorId="2" shapeId="0" xr:uid="{785D315C-EB53-42A1-A495-EF7EA88212BE}">
+    <comment ref="W4" authorId="2" shapeId="0" xr:uid="{785D315C-EB53-42A1-A495-EF7EA88212BE}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="207">
   <si>
     <t>PIDINST Batch Instrument Upload Template (single-sheet, arrays via repeated rows)</t>
   </si>
@@ -218,9 +218,6 @@
   </si>
   <si>
     <t>Example description</t>
-  </si>
-  <si>
-    <t>2026-01-15</t>
   </si>
   <si>
     <t>URL</t>
@@ -683,6 +680,15 @@
   </si>
   <si>
     <t>Period of Activity</t>
+  </si>
+  <si>
+    <t>2020-01-15</t>
+  </si>
+  <si>
+    <t>PKG_ID</t>
+  </si>
+  <si>
+    <t>Database ID of the record. Only usable for UPDATE purpose. For CREATE, leave it empty</t>
   </si>
 </sst>
 </file>
@@ -1005,6 +1011,24 @@
     <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1023,6 +1047,33 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1032,39 +1083,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1073,18 +1091,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1285,13 +1291,13 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="O4" dT="2026-02-24T04:50:16.07" personId="{008F8B26-F0D6-41D1-B35B-B7382B629FC0}" id="{3449D359-B9EE-4FE3-8BA1-8E90EA1E9711}">
+  <threadedComment ref="P4" dT="2026-02-24T04:50:16.07" personId="{008F8B26-F0D6-41D1-B35B-B7382B629FC0}" id="{3449D359-B9EE-4FE3-8BA1-8E90EA1E9711}">
     <text>The first record on instrument type will also be picked for resourceType. This is just for mapping to DataCite</text>
   </threadedComment>
-  <threadedComment ref="Q4" dT="2026-02-24T04:51:31.05" personId="{008F8B26-F0D6-41D1-B35B-B7382B629FC0}" id="{EB2AA444-AB45-471F-B2D2-3762B9440EA1}">
+  <threadedComment ref="R4" dT="2026-02-24T04:51:31.05" personId="{008F8B26-F0D6-41D1-B35B-B7382B629FC0}" id="{EB2AA444-AB45-471F-B2D2-3762B9440EA1}">
     <text>Use this block for resources that are not registered in our Instrument Registry (e.g. related documents or datasets)</text>
   </threadedComment>
-  <threadedComment ref="V4" dT="2026-02-24T04:52:30.33" personId="{008F8B26-F0D6-41D1-B35B-B7382B629FC0}" id="{785D315C-EB53-42A1-A495-EF7EA88212BE}">
+  <threadedComment ref="W4" dT="2026-02-24T04:52:30.33" personId="{008F8B26-F0D6-41D1-B35B-B7382B629FC0}" id="{785D315C-EB53-42A1-A495-EF7EA88212BE}">
     <text xml:space="preserve">Use this to link an existing instrument in our system to this instrument. You can either provide the ID for the instrument (easiest and safest) or You can provide a combo of (manf, model, sn) and we will search and find the related instrument
 </text>
   </threadedComment>
@@ -1300,673 +1306,683 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AV9"/>
+  <dimension ref="A1:AW9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="3" width="23.7109375" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="20.7109375" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="24" customWidth="1"/>
-    <col min="13" max="13" width="39.7109375" style="15" customWidth="1"/>
-    <col min="14" max="14" width="22" customWidth="1"/>
-    <col min="15" max="15" width="21.85546875" customWidth="1"/>
-    <col min="16" max="16" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24" customWidth="1"/>
-    <col min="18" max="20" width="18" customWidth="1"/>
-    <col min="21" max="21" width="22" customWidth="1"/>
-    <col min="22" max="22" width="20.5703125" customWidth="1"/>
-    <col min="23" max="23" width="14.42578125" customWidth="1"/>
-    <col min="24" max="24" width="14.140625" customWidth="1"/>
-    <col min="25" max="25" width="22" customWidth="1"/>
-    <col min="26" max="26" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="24.7109375" customWidth="1"/>
-    <col min="28" max="28" width="38" customWidth="1"/>
-    <col min="29" max="29" width="31.85546875" customWidth="1"/>
-    <col min="30" max="30" width="16" customWidth="1"/>
-    <col min="31" max="32" width="22" customWidth="1"/>
-    <col min="33" max="33" width="20" customWidth="1"/>
-    <col min="34" max="36" width="18" customWidth="1"/>
-    <col min="37" max="37" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="39" max="42" width="10.28515625" customWidth="1"/>
-    <col min="43" max="43" width="10" customWidth="1"/>
-    <col min="44" max="44" width="46.28515625" customWidth="1"/>
-    <col min="45" max="45" width="22" customWidth="1"/>
-    <col min="46" max="46" width="12.140625" customWidth="1"/>
-    <col min="47" max="47" width="18.28515625" customWidth="1"/>
-    <col min="48" max="48" width="28.140625" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" customWidth="1"/>
+    <col min="3" max="4" width="23.7109375" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="12" width="22" customWidth="1"/>
+    <col min="13" max="13" width="24" customWidth="1"/>
+    <col min="14" max="14" width="39.7109375" style="15" customWidth="1"/>
+    <col min="15" max="15" width="22" customWidth="1"/>
+    <col min="16" max="16" width="21.85546875" customWidth="1"/>
+    <col min="17" max="17" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24" customWidth="1"/>
+    <col min="19" max="21" width="18" customWidth="1"/>
+    <col min="22" max="22" width="22" customWidth="1"/>
+    <col min="23" max="23" width="20.5703125" customWidth="1"/>
+    <col min="24" max="24" width="14.42578125" customWidth="1"/>
+    <col min="25" max="25" width="14.140625" customWidth="1"/>
+    <col min="26" max="26" width="22" customWidth="1"/>
+    <col min="27" max="27" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="24.7109375" customWidth="1"/>
+    <col min="29" max="29" width="38" customWidth="1"/>
+    <col min="30" max="30" width="31.85546875" customWidth="1"/>
+    <col min="31" max="31" width="16" customWidth="1"/>
+    <col min="32" max="33" width="22" customWidth="1"/>
+    <col min="34" max="34" width="20" customWidth="1"/>
+    <col min="35" max="37" width="18" customWidth="1"/>
+    <col min="38" max="38" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="40" max="43" width="10.28515625" customWidth="1"/>
+    <col min="44" max="44" width="10" customWidth="1"/>
+    <col min="45" max="45" width="46.28515625" customWidth="1"/>
+    <col min="46" max="46" width="22" customWidth="1"/>
+    <col min="47" max="47" width="12.140625" customWidth="1"/>
+    <col min="48" max="48" width="18.28515625" customWidth="1"/>
+    <col min="49" max="49" width="28.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:49" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:48" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="B1" s="6"/>
+    </row>
+    <row r="2" spans="1:49" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="23"/>
+      <c r="S2" s="23"/>
+      <c r="T2" s="23"/>
+      <c r="U2" s="23"/>
+      <c r="V2" s="23"/>
+      <c r="W2" s="23"/>
+      <c r="X2" s="23"/>
+      <c r="Y2" s="23"/>
+      <c r="Z2" s="23"/>
+      <c r="AA2" s="23"/>
+      <c r="AB2" s="23"/>
+      <c r="AC2" s="23"/>
+      <c r="AD2" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="17"/>
-      <c r="Q2" s="17"/>
-      <c r="R2" s="17"/>
-      <c r="S2" s="17"/>
-      <c r="T2" s="17"/>
-      <c r="U2" s="17"/>
-      <c r="V2" s="17"/>
-      <c r="W2" s="17"/>
-      <c r="X2" s="17"/>
-      <c r="Y2" s="17"/>
-      <c r="Z2" s="17"/>
-      <c r="AA2" s="17"/>
-      <c r="AB2" s="17"/>
-      <c r="AC2" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="AD2" s="22"/>
-      <c r="AE2" s="22"/>
-      <c r="AF2" s="22"/>
-      <c r="AG2" s="22"/>
-      <c r="AH2" s="22"/>
-      <c r="AI2" s="22"/>
-      <c r="AJ2" s="22"/>
-      <c r="AK2" s="22"/>
-      <c r="AL2" s="22"/>
-      <c r="AM2" s="22"/>
-      <c r="AN2" s="22"/>
-      <c r="AO2" s="22"/>
-      <c r="AP2" s="22"/>
-      <c r="AQ2" s="22"/>
-      <c r="AR2" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="AS2" s="22"/>
-      <c r="AT2" s="22"/>
-      <c r="AU2" s="22"/>
-      <c r="AV2" s="22"/>
-    </row>
-    <row r="3" spans="1:48" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AE2" s="28"/>
+      <c r="AF2" s="28"/>
+      <c r="AG2" s="28"/>
+      <c r="AH2" s="28"/>
+      <c r="AI2" s="28"/>
+      <c r="AJ2" s="28"/>
+      <c r="AK2" s="28"/>
+      <c r="AL2" s="28"/>
+      <c r="AM2" s="28"/>
+      <c r="AN2" s="28"/>
+      <c r="AO2" s="28"/>
+      <c r="AP2" s="28"/>
+      <c r="AQ2" s="28"/>
+      <c r="AR2" s="28"/>
+      <c r="AS2" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="AT2" s="28"/>
+      <c r="AU2" s="28"/>
+      <c r="AV2" s="28"/>
+      <c r="AW2" s="28"/>
+    </row>
+    <row r="3" spans="1:49" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
-      <c r="B3" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="34" t="s">
+      <c r="B3" s="38" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="M3" s="36"/>
+      <c r="N3" s="36"/>
+      <c r="O3" s="36"/>
+      <c r="P3" s="36"/>
+      <c r="Q3" s="36"/>
+      <c r="R3" s="36"/>
+      <c r="S3" s="36"/>
+      <c r="T3" s="36"/>
+      <c r="U3" s="36"/>
+      <c r="V3" s="36"/>
+      <c r="W3" s="36"/>
+      <c r="X3" s="36"/>
+      <c r="Y3" s="36"/>
+      <c r="Z3" s="36"/>
+      <c r="AA3" s="36"/>
+      <c r="AB3" s="36"/>
+      <c r="AC3" s="37"/>
+      <c r="AD3" s="41" t="s">
         <v>136</v>
       </c>
-      <c r="L3" s="35"/>
-      <c r="M3" s="35"/>
-      <c r="N3" s="35"/>
-      <c r="O3" s="35"/>
-      <c r="P3" s="35"/>
-      <c r="Q3" s="35"/>
-      <c r="R3" s="35"/>
-      <c r="S3" s="35"/>
-      <c r="T3" s="35"/>
-      <c r="U3" s="35"/>
-      <c r="V3" s="35"/>
-      <c r="W3" s="35"/>
-      <c r="X3" s="35"/>
-      <c r="Y3" s="35"/>
-      <c r="Z3" s="35"/>
-      <c r="AA3" s="35"/>
-      <c r="AB3" s="36"/>
-      <c r="AC3" s="37" t="s">
-        <v>137</v>
-      </c>
-      <c r="AD3" s="38"/>
-      <c r="AE3" s="38"/>
-      <c r="AF3" s="38"/>
-      <c r="AG3" s="38"/>
-      <c r="AH3" s="38"/>
-      <c r="AI3" s="38"/>
-      <c r="AJ3" s="38"/>
-      <c r="AK3" s="38"/>
-      <c r="AL3" s="38"/>
-      <c r="AM3" s="38"/>
-      <c r="AN3" s="38"/>
-      <c r="AO3" s="38"/>
-      <c r="AP3" s="38"/>
-      <c r="AQ3" s="39"/>
-      <c r="AR3" s="20" t="s">
-        <v>142</v>
-      </c>
-      <c r="AS3" s="21"/>
-      <c r="AT3" s="21"/>
-      <c r="AU3" s="21"/>
-      <c r="AV3" s="21"/>
-    </row>
-    <row r="4" spans="1:48" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AE3" s="42"/>
+      <c r="AF3" s="42"/>
+      <c r="AG3" s="42"/>
+      <c r="AH3" s="42"/>
+      <c r="AI3" s="42"/>
+      <c r="AJ3" s="42"/>
+      <c r="AK3" s="42"/>
+      <c r="AL3" s="42"/>
+      <c r="AM3" s="42"/>
+      <c r="AN3" s="42"/>
+      <c r="AO3" s="42"/>
+      <c r="AP3" s="42"/>
+      <c r="AQ3" s="42"/>
+      <c r="AR3" s="43"/>
+      <c r="AS3" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="AT3" s="27"/>
+      <c r="AU3" s="27"/>
+      <c r="AV3" s="27"/>
+      <c r="AW3" s="27"/>
+    </row>
+    <row r="4" spans="1:49" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="E4" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="D4" s="13" t="s">
+      <c r="F4" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="E4" s="26" t="s">
+      <c r="G4" s="30"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="F4" s="27"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="26" t="s">
+      <c r="J4" s="30"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="29" t="s">
+      <c r="M4" s="21"/>
+      <c r="N4" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="L4" s="30"/>
-      <c r="M4" s="29" t="s">
+      <c r="O4" s="22"/>
+      <c r="P4" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="N4" s="40"/>
-      <c r="O4" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="P4" s="30"/>
-      <c r="Q4" s="41" t="s">
+      <c r="Q4" s="21"/>
+      <c r="R4" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="S4" s="18"/>
+      <c r="T4" s="18"/>
+      <c r="U4" s="18"/>
+      <c r="V4" s="19"/>
+      <c r="W4" s="20" t="s">
         <v>197</v>
       </c>
-      <c r="R4" s="42"/>
-      <c r="S4" s="42"/>
-      <c r="T4" s="42"/>
-      <c r="U4" s="43"/>
-      <c r="V4" s="29" t="s">
-        <v>198</v>
-      </c>
-      <c r="W4" s="30"/>
-      <c r="X4" s="30"/>
-      <c r="Y4" s="30"/>
-      <c r="Z4" s="29" t="s">
+      <c r="X4" s="21"/>
+      <c r="Y4" s="21"/>
+      <c r="Z4" s="21"/>
+      <c r="AA4" s="20" t="s">
+        <v>126</v>
+      </c>
+      <c r="AB4" s="21"/>
+      <c r="AC4" s="22"/>
+      <c r="AD4" s="32" t="s">
+        <v>134</v>
+      </c>
+      <c r="AE4" s="33"/>
+      <c r="AF4" s="33"/>
+      <c r="AG4" s="34"/>
+      <c r="AH4" s="32" t="s">
+        <v>126</v>
+      </c>
+      <c r="AI4" s="34"/>
+      <c r="AJ4" s="32" t="s">
         <v>127</v>
       </c>
-      <c r="AA4" s="30"/>
-      <c r="AB4" s="40"/>
-      <c r="AC4" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="AD4" s="32"/>
-      <c r="AE4" s="32"/>
-      <c r="AF4" s="33"/>
-      <c r="AG4" s="31" t="s">
-        <v>127</v>
-      </c>
-      <c r="AH4" s="33"/>
-      <c r="AI4" s="31" t="s">
-        <v>128</v>
-      </c>
-      <c r="AJ4" s="32"/>
-      <c r="AK4" s="32"/>
-      <c r="AL4" s="32"/>
-      <c r="AM4" s="32"/>
-      <c r="AN4" s="32"/>
-      <c r="AO4" s="32"/>
-      <c r="AP4" s="32"/>
+      <c r="AK4" s="33"/>
+      <c r="AL4" s="33"/>
+      <c r="AM4" s="33"/>
+      <c r="AN4" s="33"/>
+      <c r="AO4" s="33"/>
+      <c r="AP4" s="33"/>
       <c r="AQ4" s="33"/>
-      <c r="AR4" s="18" t="s">
-        <v>141</v>
-      </c>
-      <c r="AS4" s="19"/>
-      <c r="AT4" s="19"/>
-      <c r="AU4" s="19"/>
-      <c r="AV4" s="19"/>
-    </row>
-    <row r="5" spans="1:48" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AR4" s="34"/>
+      <c r="AS4" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="AT4" s="25"/>
+      <c r="AU4" s="25"/>
+      <c r="AV4" s="25"/>
+      <c r="AW4" s="25"/>
+    </row>
+    <row r="5" spans="1:49" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="M5" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="M5" s="16" t="s">
+      <c r="N5" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="N5" s="10" t="s">
+      <c r="O5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="P5" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q5" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="P5" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="Q5" s="10" t="s">
+      <c r="R5" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="S5" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="R5" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="S5" s="10" t="s">
-        <v>124</v>
-      </c>
       <c r="T5" s="10" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="U5" s="10" t="s">
         <v>125</v>
       </c>
       <c r="V5" s="10" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="W5" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="X5" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="Y5" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="X5" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="Y5" s="10" t="s">
+      <c r="Z5" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="AA5" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="AB5" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="AC5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD5" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="AE5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="AH5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="AI5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="AJ5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AK5" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="AL5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="AM5" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AN5" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="AO5" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="AP5" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="AQ5" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="AR5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="AS5" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="AT5" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="AU5" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="AV5" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="AW5" s="11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:49" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="U6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="Z6" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="Z5" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="AA5" s="1" t="s">
+      <c r="AA6" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="AB5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="AC5" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="AD5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="AE5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="AF5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="AG5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="AH5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="AI5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="AJ5" s="1" t="s">
+      <c r="AB6" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="AC6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AD6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="AE6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="AF6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="AG6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AH6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AI6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AJ6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AK6" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="AK5" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="AL5" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="AM5" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="AN5" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="AO5" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="AP5" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="AQ5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="AR5" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="AS5" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="AT5" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="AU5" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="AV5" s="11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:48" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="O6" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="P6" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="Q6" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R6" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="S6" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="T6" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="U6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="V6" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="W6" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="X6" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="Y6" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="Z6" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="AA6" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="AB6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AC6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AD6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AE6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AF6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AG6" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="AH6" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="AI6" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="AJ6" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="AK6" s="2" t="s">
+      <c r="AL6" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="AM6" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="AN6" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="AL6" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="AM6" s="2" t="s">
+      <c r="AO6" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="AN6" s="2" t="s">
+      <c r="AP6" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AO6" s="2" t="s">
+      <c r="AQ6" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AP6" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="AQ6" s="2" t="s">
+      <c r="AR6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AR6" s="12" t="s">
+      <c r="AS6" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="AT6" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="AS6" s="12" t="s">
+      <c r="AU6" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="AT6" s="12" t="s">
+      <c r="AV6" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="AU6" s="12" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="7" spans="1:48" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>47</v>
       </c>
-      <c r="C7" t="s">
-        <v>171</v>
-      </c>
       <c r="D7" t="s">
+        <v>170</v>
+      </c>
+      <c r="E7" t="s">
+        <v>188</v>
+      </c>
+      <c r="F7" t="s">
+        <v>130</v>
+      </c>
+      <c r="G7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" t="s">
+        <v>50</v>
+      </c>
+      <c r="I7" t="s">
+        <v>201</v>
+      </c>
+      <c r="J7" t="s">
+        <v>54</v>
+      </c>
+      <c r="K7" t="s">
+        <v>50</v>
+      </c>
+      <c r="L7" t="s">
         <v>189</v>
       </c>
-      <c r="E7" t="s">
-        <v>131</v>
-      </c>
-      <c r="F7" t="s">
-        <v>50</v>
-      </c>
-      <c r="G7" t="s">
-        <v>50</v>
-      </c>
-      <c r="H7" t="s">
-        <v>202</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="M7" t="s">
+        <v>48</v>
+      </c>
+      <c r="N7" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="O7" t="s">
+        <v>128</v>
+      </c>
+      <c r="P7" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>190</v>
+      </c>
+      <c r="R7" t="s">
         <v>55</v>
       </c>
-      <c r="J7" t="s">
-        <v>50</v>
-      </c>
-      <c r="K7" t="s">
-        <v>190</v>
-      </c>
-      <c r="L7" t="s">
-        <v>48</v>
-      </c>
-      <c r="M7" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="N7" t="s">
-        <v>129</v>
-      </c>
-      <c r="O7" t="s">
-        <v>193</v>
-      </c>
-      <c r="P7" t="s">
+      <c r="S7" t="s">
+        <v>56</v>
+      </c>
+      <c r="T7" t="s">
+        <v>57</v>
+      </c>
+      <c r="U7" t="s">
+        <v>58</v>
+      </c>
+      <c r="V7" t="s">
+        <v>50</v>
+      </c>
+      <c r="X7" t="s">
+        <v>188</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>200</v>
+      </c>
+      <c r="Z7">
+        <v>1</v>
+      </c>
+      <c r="AA7" t="s">
         <v>191</v>
       </c>
-      <c r="Q7" t="s">
-        <v>56</v>
-      </c>
-      <c r="R7" t="s">
-        <v>57</v>
-      </c>
-      <c r="S7" t="s">
-        <v>58</v>
-      </c>
-      <c r="T7" t="s">
+      <c r="AB7" t="s">
+        <v>167</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>158</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>61</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AJ7" t="s">
         <v>59</v>
       </c>
-      <c r="U7" t="s">
-        <v>50</v>
-      </c>
-      <c r="W7" t="s">
-        <v>189</v>
-      </c>
-      <c r="X7" t="s">
-        <v>201</v>
-      </c>
-      <c r="Y7">
-        <v>1</v>
-      </c>
-      <c r="Z7" t="s">
-        <v>192</v>
-      </c>
-      <c r="AA7" t="s">
-        <v>168</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>51</v>
-      </c>
-      <c r="AC7" t="s">
-        <v>159</v>
-      </c>
-      <c r="AD7" t="s">
-        <v>50</v>
-      </c>
-      <c r="AE7" t="s">
-        <v>50</v>
-      </c>
-      <c r="AF7" t="s">
-        <v>50</v>
-      </c>
-      <c r="AG7" t="s">
-        <v>62</v>
-      </c>
-      <c r="AH7" t="s">
-        <v>50</v>
-      </c>
-      <c r="AI7" t="s">
-        <v>60</v>
-      </c>
-      <c r="AJ7" t="s">
-        <v>99</v>
-      </c>
-      <c r="AK7">
+      <c r="AK7" t="s">
+        <v>98</v>
+      </c>
+      <c r="AL7">
         <v>115.86</v>
       </c>
-      <c r="AL7">
+      <c r="AM7">
         <v>-31.952200000000001</v>
       </c>
-      <c r="AQ7">
+      <c r="AR7">
         <v>4326</v>
       </c>
-      <c r="AR7" t="s">
-        <v>156</v>
-      </c>
       <c r="AS7" t="s">
+        <v>155</v>
+      </c>
+      <c r="AT7" t="s">
+        <v>150</v>
+      </c>
+      <c r="AU7" t="s">
+        <v>147</v>
+      </c>
+      <c r="AV7" t="s">
         <v>151</v>
       </c>
-      <c r="AT7" t="s">
-        <v>148</v>
-      </c>
-      <c r="AU7" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="8" spans="1:48" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1</v>
       </c>
-      <c r="B8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C8" t="s">
         <v>50</v>
       </c>
       <c r="E8" t="s">
@@ -1979,27 +1995,27 @@
         <v>50</v>
       </c>
       <c r="H8" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="I8" t="s">
-        <v>97</v>
-      </c>
-      <c r="K8" t="s">
-        <v>50</v>
+        <v>62</v>
+      </c>
+      <c r="J8" t="s">
+        <v>96</v>
       </c>
       <c r="L8" t="s">
         <v>50</v>
       </c>
-      <c r="M8" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="N8" t="s">
+      <c r="M8" t="s">
+        <v>50</v>
+      </c>
+      <c r="N8" s="15" t="s">
         <v>50</v>
       </c>
       <c r="O8" t="s">
         <v>50</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="P8" t="s">
         <v>50</v>
       </c>
       <c r="R8" t="s">
@@ -2014,7 +2030,7 @@
       <c r="U8" t="s">
         <v>50</v>
       </c>
-      <c r="AB8" t="s">
+      <c r="V8" t="s">
         <v>50</v>
       </c>
       <c r="AC8" t="s">
@@ -2038,63 +2054,66 @@
       <c r="AI8" t="s">
         <v>50</v>
       </c>
-      <c r="AL8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AQ8" t="s">
+      <c r="AJ8" t="s">
+        <v>50</v>
+      </c>
+      <c r="AM8" t="s">
         <v>50</v>
       </c>
       <c r="AR8" t="s">
-        <v>157</v>
+        <v>50</v>
       </c>
       <c r="AS8" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="AT8" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="AU8" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="9" spans="1:48" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+      <c r="AV8" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1</v>
       </c>
-      <c r="AR9" t="s">
-        <v>158</v>
-      </c>
       <c r="AS9" t="s">
+        <v>157</v>
+      </c>
+      <c r="AT9" t="s">
+        <v>153</v>
+      </c>
+      <c r="AU9" t="s">
+        <v>148</v>
+      </c>
+      <c r="AV9" t="s">
         <v>154</v>
-      </c>
-      <c r="AT9" t="s">
-        <v>149</v>
-      </c>
-      <c r="AU9" t="s">
-        <v>155</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="Q4:U4"/>
-    <mergeCell ref="V4:Y4"/>
-    <mergeCell ref="Z4:AB4"/>
-    <mergeCell ref="A2:AB2"/>
-    <mergeCell ref="AR4:AV4"/>
-    <mergeCell ref="AR3:AV3"/>
-    <mergeCell ref="AR2:AV2"/>
-    <mergeCell ref="AC2:AQ2"/>
-    <mergeCell ref="B3:J3"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="AC4:AF4"/>
-    <mergeCell ref="AG4:AH4"/>
-    <mergeCell ref="AI4:AQ4"/>
-    <mergeCell ref="K3:AB3"/>
-    <mergeCell ref="AC3:AQ3"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="AD3:AR3"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="R4:V4"/>
+    <mergeCell ref="W4:Z4"/>
+    <mergeCell ref="AA4:AC4"/>
+    <mergeCell ref="A2:AC2"/>
+    <mergeCell ref="AS4:AW4"/>
+    <mergeCell ref="AS3:AW3"/>
+    <mergeCell ref="AS2:AW2"/>
+    <mergeCell ref="AD2:AR2"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="AD4:AG4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AJ4:AR4"/>
+    <mergeCell ref="L3:AC3"/>
+    <mergeCell ref="B3:K3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -2109,55 +2128,55 @@
           <x14:formula1>
             <xm:f>_lists!$A$52:$A$54</xm:f>
           </x14:formula1>
-          <xm:sqref>I7:I1048576</xm:sqref>
+          <xm:sqref>J7:J1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D8B9F839-0BDE-4FD4-B802-1C94BF58BC01}">
           <x14:formula1>
             <xm:f>_lists!$A$36:$A$39</xm:f>
           </x14:formula1>
-          <xm:sqref>S7:S1048576</xm:sqref>
+          <xm:sqref>T7:T1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A7430D0B-6D07-4C77-B74B-4D22515A3B08}">
           <x14:formula1>
             <xm:f>_lists!$A$43:$A$46</xm:f>
           </x14:formula1>
-          <xm:sqref>T8:T1048576</xm:sqref>
+          <xm:sqref>U8:U1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D0553167-78DD-4985-947D-26B90EED3A92}">
           <x14:formula1>
             <xm:f>_lists!$A$43:$A$48</xm:f>
           </x14:formula1>
-          <xm:sqref>T7</xm:sqref>
+          <xm:sqref>U7</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A0FE94E2-3A12-46E7-AC69-5BD022234573}">
           <x14:formula1>
             <xm:f>_lists!$A$14:$A$33</xm:f>
           </x14:formula1>
-          <xm:sqref>R7:R1048576</xm:sqref>
+          <xm:sqref>S7:S1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B06767BB-3B31-45E1-A681-98128DFD18C8}">
           <x14:formula1>
             <xm:f>_lists!$A$75:$A$76</xm:f>
           </x14:formula1>
-          <xm:sqref>AT7:AT1048576</xm:sqref>
+          <xm:sqref>AU7:AU1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{92A0783E-8438-44B7-8D64-4FE7175FA9FB}">
           <x14:formula1>
             <xm:f>_lists!$A$79:$A$81</xm:f>
           </x14:formula1>
-          <xm:sqref>C7:C1048576</xm:sqref>
+          <xm:sqref>D7:D1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8E91E68E-1DCC-47C2-8753-4026B09E5314}">
           <x14:formula1>
             <xm:f>_lists!$A$84:$A$86</xm:f>
           </x14:formula1>
-          <xm:sqref>AJ7:AJ1048576</xm:sqref>
+          <xm:sqref>AK7:AK1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{56BC94EC-09BC-4572-B5EA-F8DA94792981}">
           <x14:formula1>
             <xm:f>_lists!$A$70:$A$72</xm:f>
           </x14:formula1>
-          <xm:sqref>N7:N1048576</xm:sqref>
+          <xm:sqref>O7:O1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2185,12 +2204,12 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
@@ -2200,27 +2219,27 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -2230,102 +2249,102 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
@@ -2335,22 +2354,22 @@
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
@@ -2360,37 +2379,37 @@
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
@@ -2400,17 +2419,17 @@
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
@@ -2420,12 +2439,12 @@
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
@@ -2435,12 +2454,12 @@
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
@@ -2450,17 +2469,17 @@
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
@@ -2470,72 +2489,72 @@
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -2558,12 +2577,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -2576,6 +2595,81 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
+      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
+      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
+    </_dlc_DocIdUrl>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C458252014B43B48B36D6FD06F31079C" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8411b2fcd13e9c262f801c2de01d8359">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9357ce84-a672-4584-8ddb-e5b553dfe263" xmlns:ns3="f66f598c-5a54-48fa-b12a-3e2e658c8d92" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7559adb2811d00dbbd5f4bbaad764c99" ns2:_="" ns3:_="">
     <xsd:import namespace="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
@@ -2837,82 +2931,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
-      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
-      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
-    </_dlc_DocIdUrl>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
+    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70706F67-F4D0-436B-9C39-1388BCD46E53}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2929,31 +2975,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
-    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
#94: enhancing GCMD taxonomy search.
</commit_message>
<xml_diff>
--- a/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
+++ b/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Drive_D\projects\avre\apps\PIDINST\AuScope-instrument-registry\ckan_batch\src\ckan_batch\reader\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B29D50-AA81-4EFD-92E0-799103CE51F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8534A0A-54AC-4895-9665-B63F2F733C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30840" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instruments" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="180">
   <si>
     <t>PIDINST Batch Instrument Upload Template (single-sheet, arrays via repeated rows)</t>
   </si>
@@ -205,21 +205,9 @@
     <t>Acknowledgements.</t>
   </si>
   <si>
-    <t>Example Instrument</t>
-  </si>
-  <si>
-    <t>contact@example.org</t>
-  </si>
-  <si>
     <t>HostingInstitution</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Example description</t>
-  </si>
-  <si>
     <t>URL</t>
   </si>
   <si>
@@ -229,9 +217,6 @@
     <t>SerialNumber</t>
   </si>
   <si>
-    <t>10.1234/example.doi</t>
-  </si>
-  <si>
     <t>DOI</t>
   </si>
   <si>
@@ -241,16 +226,7 @@
     <t>Collects</t>
   </si>
   <si>
-    <t>Perth, WA</t>
-  </si>
-  <si>
     <t>true</t>
-  </si>
-  <si>
-    <t>mineral,geochem</t>
-  </si>
-  <si>
-    <t>ALT-123</t>
   </si>
   <si>
     <t>Other</t>
@@ -460,9 +436,6 @@
     <t>Decommissioned</t>
   </si>
   <si>
-    <t>CGS-T</t>
-  </si>
-  <si>
     <t>Id*</t>
   </si>
   <si>
@@ -520,33 +493,6 @@
     <t>Path</t>
   </si>
   <si>
-    <t>cover image</t>
-  </si>
-  <si>
-    <t>jpg</t>
-  </si>
-  <si>
-    <t>image</t>
-  </si>
-  <si>
-    <t>data</t>
-  </si>
-  <si>
-    <t>csv</t>
-  </si>
-  <si>
-    <t>~\CSIRO\AuScope AVRE - Persistent ID for Instruments (PIDINST)\data\accessories-for-mineralogy-microscopes.jpg</t>
-  </si>
-  <si>
-    <t>~\CSIRO\AuScope AVRE - Persistent ID for Instruments (PIDINST)\data\MDU-Hylogger-drill-core.jpg</t>
-  </si>
-  <si>
-    <t>~\Downloads\maia-statistics-2026-03-03T04-12-50.csv</t>
-  </si>
-  <si>
-    <t>AuScope</t>
-  </si>
-  <si>
     <t>instrumentTypeGCMD</t>
   </si>
   <si>
@@ -571,9 +517,6 @@
     <t>Measured variables from our own taxonomies (For multiple entries, separate by ",").</t>
   </si>
   <si>
-    <t>Magnetic Field</t>
-  </si>
-  <si>
     <t>Class*</t>
   </si>
   <si>
@@ -634,21 +577,6 @@
     <t>max_lat</t>
   </si>
   <si>
-    <t>Phoenix Geophysics</t>
-  </si>
-  <si>
-    <t>Curtin Hub for Immersive Visualisation and eResearch</t>
-  </si>
-  <si>
-    <t>Magneto-test</t>
-  </si>
-  <si>
-    <t>temperature,pressure</t>
-  </si>
-  <si>
-    <t>MICROSCOPES</t>
-  </si>
-  <si>
     <t>Associated DOI for the instrument</t>
   </si>
   <si>
@@ -670,19 +598,10 @@
     <t>Alternate Identifier of the instrument (just provide the code)</t>
   </si>
   <si>
-    <t>MTU-5C</t>
-  </si>
-  <si>
-    <t>SN-111111</t>
-  </si>
-  <si>
     <t>Relevant date in YYYY or YYYY-MM or YYYY-MM-DD. For Coverage, you can provide range dates according to RKMS-ISO8601</t>
   </si>
   <si>
     <t>Period of Activity</t>
-  </si>
-  <si>
-    <t>2020-01-15</t>
   </si>
   <si>
     <t>PKG_ID</t>
@@ -1011,6 +930,24 @@
     <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1020,15 +957,6 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1081,15 +1009,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1306,7 +1225,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AW9"/>
+  <dimension ref="A1:AW6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1357,243 +1276,243 @@
       <c r="B1" s="6"/>
     </row>
     <row r="2" spans="1:49" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="23"/>
-      <c r="Z2" s="23"/>
-      <c r="AA2" s="23"/>
-      <c r="AB2" s="23"/>
-      <c r="AC2" s="23"/>
-      <c r="AD2" s="28" t="s">
-        <v>122</v>
-      </c>
-      <c r="AE2" s="28"/>
-      <c r="AF2" s="28"/>
-      <c r="AG2" s="28"/>
-      <c r="AH2" s="28"/>
-      <c r="AI2" s="28"/>
-      <c r="AJ2" s="28"/>
-      <c r="AK2" s="28"/>
-      <c r="AL2" s="28"/>
-      <c r="AM2" s="28"/>
-      <c r="AN2" s="28"/>
-      <c r="AO2" s="28"/>
-      <c r="AP2" s="28"/>
-      <c r="AQ2" s="28"/>
-      <c r="AR2" s="28"/>
-      <c r="AS2" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="AT2" s="28"/>
-      <c r="AU2" s="28"/>
-      <c r="AV2" s="28"/>
-      <c r="AW2" s="28"/>
+      <c r="A2" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26"/>
+      <c r="R2" s="26"/>
+      <c r="S2" s="26"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="26"/>
+      <c r="V2" s="26"/>
+      <c r="W2" s="26"/>
+      <c r="X2" s="26"/>
+      <c r="Y2" s="26"/>
+      <c r="Z2" s="26"/>
+      <c r="AA2" s="26"/>
+      <c r="AB2" s="26"/>
+      <c r="AC2" s="26"/>
+      <c r="AD2" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="AE2" s="31"/>
+      <c r="AF2" s="31"/>
+      <c r="AG2" s="31"/>
+      <c r="AH2" s="31"/>
+      <c r="AI2" s="31"/>
+      <c r="AJ2" s="31"/>
+      <c r="AK2" s="31"/>
+      <c r="AL2" s="31"/>
+      <c r="AM2" s="31"/>
+      <c r="AN2" s="31"/>
+      <c r="AO2" s="31"/>
+      <c r="AP2" s="31"/>
+      <c r="AQ2" s="31"/>
+      <c r="AR2" s="31"/>
+      <c r="AS2" s="31" t="s">
+        <v>132</v>
+      </c>
+      <c r="AT2" s="31"/>
+      <c r="AU2" s="31"/>
+      <c r="AV2" s="31"/>
+      <c r="AW2" s="31"/>
     </row>
     <row r="3" spans="1:49" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
-      <c r="B3" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="39"/>
-      <c r="G3" s="39"/>
-      <c r="H3" s="39"/>
-      <c r="I3" s="39"/>
-      <c r="J3" s="39"/>
-      <c r="K3" s="40"/>
-      <c r="L3" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="M3" s="36"/>
-      <c r="N3" s="36"/>
-      <c r="O3" s="36"/>
-      <c r="P3" s="36"/>
-      <c r="Q3" s="36"/>
-      <c r="R3" s="36"/>
-      <c r="S3" s="36"/>
-      <c r="T3" s="36"/>
-      <c r="U3" s="36"/>
-      <c r="V3" s="36"/>
-      <c r="W3" s="36"/>
-      <c r="X3" s="36"/>
-      <c r="Y3" s="36"/>
-      <c r="Z3" s="36"/>
-      <c r="AA3" s="36"/>
-      <c r="AB3" s="36"/>
-      <c r="AC3" s="37"/>
-      <c r="AD3" s="41" t="s">
-        <v>136</v>
-      </c>
-      <c r="AE3" s="42"/>
-      <c r="AF3" s="42"/>
-      <c r="AG3" s="42"/>
-      <c r="AH3" s="42"/>
-      <c r="AI3" s="42"/>
-      <c r="AJ3" s="42"/>
-      <c r="AK3" s="42"/>
-      <c r="AL3" s="42"/>
-      <c r="AM3" s="42"/>
-      <c r="AN3" s="42"/>
-      <c r="AO3" s="42"/>
-      <c r="AP3" s="42"/>
-      <c r="AQ3" s="42"/>
-      <c r="AR3" s="43"/>
-      <c r="AS3" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="AT3" s="27"/>
-      <c r="AU3" s="27"/>
-      <c r="AV3" s="27"/>
-      <c r="AW3" s="27"/>
+      <c r="B3" s="41" t="s">
+        <v>124</v>
+      </c>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="43"/>
+      <c r="L3" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
+      <c r="P3" s="39"/>
+      <c r="Q3" s="39"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="39"/>
+      <c r="T3" s="39"/>
+      <c r="U3" s="39"/>
+      <c r="V3" s="39"/>
+      <c r="W3" s="39"/>
+      <c r="X3" s="39"/>
+      <c r="Y3" s="39"/>
+      <c r="Z3" s="39"/>
+      <c r="AA3" s="39"/>
+      <c r="AB3" s="39"/>
+      <c r="AC3" s="40"/>
+      <c r="AD3" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="AE3" s="18"/>
+      <c r="AF3" s="18"/>
+      <c r="AG3" s="18"/>
+      <c r="AH3" s="18"/>
+      <c r="AI3" s="18"/>
+      <c r="AJ3" s="18"/>
+      <c r="AK3" s="18"/>
+      <c r="AL3" s="18"/>
+      <c r="AM3" s="18"/>
+      <c r="AN3" s="18"/>
+      <c r="AO3" s="18"/>
+      <c r="AP3" s="18"/>
+      <c r="AQ3" s="18"/>
+      <c r="AR3" s="19"/>
+      <c r="AS3" s="29" t="s">
+        <v>132</v>
+      </c>
+      <c r="AT3" s="30"/>
+      <c r="AU3" s="30"/>
+      <c r="AV3" s="30"/>
+      <c r="AW3" s="30"/>
     </row>
     <row r="4" spans="1:49" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="9" t="s">
-        <v>205</v>
+        <v>178</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>183</v>
+        <v>164</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="F4" s="29" t="s">
-        <v>116</v>
-      </c>
-      <c r="G4" s="30"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="29" t="s">
-        <v>117</v>
-      </c>
-      <c r="J4" s="30"/>
-      <c r="K4" s="31"/>
+        <v>107</v>
+      </c>
+      <c r="F4" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="G4" s="33"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="J4" s="33"/>
+      <c r="K4" s="34"/>
       <c r="L4" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="M4" s="22"/>
+      <c r="N4" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="O4" s="21"/>
+      <c r="P4" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q4" s="22"/>
+      <c r="R4" s="23" t="s">
+        <v>172</v>
+      </c>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
+      <c r="U4" s="24"/>
+      <c r="V4" s="25"/>
+      <c r="W4" s="20" t="s">
+        <v>173</v>
+      </c>
+      <c r="X4" s="22"/>
+      <c r="Y4" s="22"/>
+      <c r="Z4" s="22"/>
+      <c r="AA4" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="M4" s="21"/>
-      <c r="N4" s="20" t="s">
+      <c r="AB4" s="22"/>
+      <c r="AC4" s="21"/>
+      <c r="AD4" s="35" t="s">
+        <v>125</v>
+      </c>
+      <c r="AE4" s="36"/>
+      <c r="AF4" s="36"/>
+      <c r="AG4" s="37"/>
+      <c r="AH4" s="35" t="s">
+        <v>118</v>
+      </c>
+      <c r="AI4" s="37"/>
+      <c r="AJ4" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="O4" s="22"/>
-      <c r="P4" s="20" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q4" s="21"/>
-      <c r="R4" s="17" t="s">
-        <v>196</v>
-      </c>
-      <c r="S4" s="18"/>
-      <c r="T4" s="18"/>
-      <c r="U4" s="18"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="20" t="s">
-        <v>197</v>
-      </c>
-      <c r="X4" s="21"/>
-      <c r="Y4" s="21"/>
-      <c r="Z4" s="21"/>
-      <c r="AA4" s="20" t="s">
-        <v>126</v>
-      </c>
-      <c r="AB4" s="21"/>
-      <c r="AC4" s="22"/>
-      <c r="AD4" s="32" t="s">
-        <v>134</v>
-      </c>
-      <c r="AE4" s="33"/>
-      <c r="AF4" s="33"/>
-      <c r="AG4" s="34"/>
-      <c r="AH4" s="32" t="s">
-        <v>126</v>
-      </c>
-      <c r="AI4" s="34"/>
-      <c r="AJ4" s="32" t="s">
-        <v>127</v>
-      </c>
-      <c r="AK4" s="33"/>
-      <c r="AL4" s="33"/>
-      <c r="AM4" s="33"/>
-      <c r="AN4" s="33"/>
-      <c r="AO4" s="33"/>
-      <c r="AP4" s="33"/>
-      <c r="AQ4" s="33"/>
-      <c r="AR4" s="34"/>
-      <c r="AS4" s="24" t="s">
-        <v>140</v>
-      </c>
-      <c r="AT4" s="25"/>
-      <c r="AU4" s="25"/>
-      <c r="AV4" s="25"/>
-      <c r="AW4" s="25"/>
+      <c r="AK4" s="36"/>
+      <c r="AL4" s="36"/>
+      <c r="AM4" s="36"/>
+      <c r="AN4" s="36"/>
+      <c r="AO4" s="36"/>
+      <c r="AP4" s="36"/>
+      <c r="AQ4" s="36"/>
+      <c r="AR4" s="37"/>
+      <c r="AS4" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="AT4" s="28"/>
+      <c r="AU4" s="28"/>
+      <c r="AV4" s="28"/>
+      <c r="AW4" s="28"/>
     </row>
     <row r="5" spans="1:49" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>2</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="N5" s="16" t="s">
         <v>5</v>
@@ -1602,43 +1521,43 @@
         <v>6</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>159</v>
+        <v>141</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="S5" s="10" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="T5" s="10" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="U5" s="10" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="V5" s="10" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="W5" s="10" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="X5" s="10" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="Y5" s="10" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="Z5" s="10" t="s">
-        <v>198</v>
+        <v>174</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>163</v>
+        <v>145</v>
       </c>
       <c r="AB5" s="1" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="AC5" s="1" t="s">
         <v>4</v>
@@ -1665,40 +1584,40 @@
         <v>17</v>
       </c>
       <c r="AK5" s="1" t="s">
-        <v>179</v>
+        <v>160</v>
       </c>
       <c r="AL5" s="1" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="AM5" s="1" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="AN5" s="1" t="s">
-        <v>184</v>
+        <v>165</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>185</v>
+        <v>166</v>
       </c>
       <c r="AP5" s="1" t="s">
-        <v>186</v>
+        <v>167</v>
       </c>
       <c r="AQ5" s="1" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="AR5" s="1" t="s">
         <v>19</v>
       </c>
       <c r="AS5" s="11" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="AT5" s="11" t="s">
         <v>2</v>
       </c>
       <c r="AU5" s="11" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="AV5" s="11" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="AW5" s="11" t="s">
         <v>4</v>
@@ -1706,16 +1625,16 @@
     </row>
     <row r="6" spans="1:49" ht="69.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>206</v>
+        <v>179</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>169</v>
+        <v>150</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>26</v>
@@ -1745,16 +1664,16 @@
         <v>25</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>202</v>
+        <v>176</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="R6" s="2" t="s">
         <v>38</v>
@@ -1772,22 +1691,22 @@
         <v>42</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>193</v>
+        <v>169</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>194</v>
+        <v>170</v>
       </c>
       <c r="Y6" s="2" t="s">
-        <v>195</v>
+        <v>171</v>
       </c>
       <c r="Z6" s="2" t="s">
-        <v>199</v>
+        <v>175</v>
       </c>
       <c r="AA6" s="2" t="s">
-        <v>165</v>
+        <v>147</v>
       </c>
       <c r="AB6" s="2" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
       <c r="AC6" s="2" t="s">
         <v>30</v>
@@ -1814,293 +1733,44 @@
         <v>43</v>
       </c>
       <c r="AK6" s="2" t="s">
-        <v>180</v>
+        <v>161</v>
       </c>
       <c r="AL6" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="AM6" s="2" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="AN6" s="2" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="AO6" s="2" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="AP6" s="2" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="AQ6" s="2" t="s">
-        <v>178</v>
+        <v>159</v>
       </c>
       <c r="AR6" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AS6" s="12" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="AT6" s="12" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="AU6" s="12" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="AV6" s="12" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="C7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" t="s">
-        <v>170</v>
-      </c>
-      <c r="E7" t="s">
-        <v>188</v>
-      </c>
-      <c r="F7" t="s">
-        <v>130</v>
-      </c>
-      <c r="G7" t="s">
-        <v>50</v>
-      </c>
-      <c r="H7" t="s">
-        <v>50</v>
-      </c>
-      <c r="I7" t="s">
-        <v>201</v>
-      </c>
-      <c r="J7" t="s">
-        <v>54</v>
-      </c>
-      <c r="K7" t="s">
-        <v>50</v>
-      </c>
-      <c r="L7" t="s">
-        <v>189</v>
-      </c>
-      <c r="M7" t="s">
-        <v>48</v>
-      </c>
-      <c r="N7" s="15" t="s">
-        <v>204</v>
-      </c>
-      <c r="O7" t="s">
-        <v>128</v>
-      </c>
-      <c r="P7" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>190</v>
-      </c>
-      <c r="R7" t="s">
-        <v>55</v>
-      </c>
-      <c r="S7" t="s">
-        <v>56</v>
-      </c>
-      <c r="T7" t="s">
-        <v>57</v>
-      </c>
-      <c r="U7" t="s">
-        <v>58</v>
-      </c>
-      <c r="V7" t="s">
-        <v>50</v>
-      </c>
-      <c r="X7" t="s">
-        <v>188</v>
-      </c>
-      <c r="Y7" t="s">
-        <v>200</v>
-      </c>
-      <c r="Z7">
-        <v>1</v>
-      </c>
-      <c r="AA7" t="s">
-        <v>191</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>167</v>
-      </c>
-      <c r="AC7" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD7" t="s">
-        <v>158</v>
-      </c>
-      <c r="AE7" t="s">
-        <v>50</v>
-      </c>
-      <c r="AF7" t="s">
-        <v>50</v>
-      </c>
-      <c r="AG7" t="s">
-        <v>50</v>
-      </c>
-      <c r="AH7" t="s">
-        <v>61</v>
-      </c>
-      <c r="AI7" t="s">
-        <v>50</v>
-      </c>
-      <c r="AJ7" t="s">
-        <v>59</v>
-      </c>
-      <c r="AK7" t="s">
-        <v>98</v>
-      </c>
-      <c r="AL7">
-        <v>115.86</v>
-      </c>
-      <c r="AM7">
-        <v>-31.952200000000001</v>
-      </c>
-      <c r="AR7">
-        <v>4326</v>
-      </c>
-      <c r="AS7" t="s">
-        <v>155</v>
-      </c>
-      <c r="AT7" t="s">
-        <v>150</v>
-      </c>
-      <c r="AU7" t="s">
-        <v>147</v>
-      </c>
-      <c r="AV7" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
-        <v>50</v>
-      </c>
-      <c r="E8" t="s">
-        <v>50</v>
-      </c>
-      <c r="F8" t="s">
-        <v>50</v>
-      </c>
-      <c r="G8" t="s">
-        <v>50</v>
-      </c>
-      <c r="H8" t="s">
-        <v>50</v>
-      </c>
-      <c r="I8" t="s">
-        <v>62</v>
-      </c>
-      <c r="J8" t="s">
-        <v>96</v>
-      </c>
-      <c r="L8" t="s">
-        <v>50</v>
-      </c>
-      <c r="M8" t="s">
-        <v>50</v>
-      </c>
-      <c r="N8" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="O8" t="s">
-        <v>50</v>
-      </c>
-      <c r="P8" t="s">
-        <v>50</v>
-      </c>
-      <c r="R8" t="s">
-        <v>50</v>
-      </c>
-      <c r="S8" t="s">
-        <v>50</v>
-      </c>
-      <c r="T8" t="s">
-        <v>50</v>
-      </c>
-      <c r="U8" t="s">
-        <v>50</v>
-      </c>
-      <c r="V8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AC8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AD8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AE8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AF8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AG8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AH8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AI8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AJ8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AM8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AR8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS8" t="s">
-        <v>156</v>
-      </c>
-      <c r="AT8" t="s">
-        <v>152</v>
-      </c>
-      <c r="AU8" t="s">
-        <v>148</v>
-      </c>
-      <c r="AV8" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>1</v>
-      </c>
-      <c r="AS9" t="s">
-        <v>157</v>
-      </c>
-      <c r="AT9" t="s">
-        <v>153</v>
-      </c>
-      <c r="AU9" t="s">
-        <v>148</v>
-      </c>
-      <c r="AV9" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="AD3:AR3"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="R4:V4"/>
-    <mergeCell ref="W4:Z4"/>
-    <mergeCell ref="AA4:AC4"/>
     <mergeCell ref="A2:AC2"/>
     <mergeCell ref="AS4:AW4"/>
     <mergeCell ref="AS3:AW3"/>
@@ -2114,6 +1784,12 @@
     <mergeCell ref="AJ4:AR4"/>
     <mergeCell ref="L3:AC3"/>
     <mergeCell ref="B3:K3"/>
+    <mergeCell ref="AD3:AR3"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="R4:V4"/>
+    <mergeCell ref="W4:Z4"/>
+    <mergeCell ref="AA4:AC4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -2199,17 +1875,17 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
@@ -2219,27 +1895,27 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -2249,102 +1925,102 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
@@ -2354,22 +2030,22 @@
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
@@ -2379,37 +2055,37 @@
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
@@ -2419,17 +2095,17 @@
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
@@ -2439,12 +2115,12 @@
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
@@ -2454,12 +2130,12 @@
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
@@ -2469,17 +2145,17 @@
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
@@ -2489,72 +2165,72 @@
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>203</v>
+        <v>177</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>170</v>
+        <v>151</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>181</v>
+        <v>162</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>182</v>
+        <v>163</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -2577,12 +2253,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2595,81 +2271,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
-      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
-      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
-    </_dlc_DocIdUrl>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C458252014B43B48B36D6FD06F31079C" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8411b2fcd13e9c262f801c2de01d8359">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9357ce84-a672-4584-8ddb-e5b553dfe263" xmlns:ns3="f66f598c-5a54-48fa-b12a-3e2e658c8d92" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7559adb2811d00dbbd5f4bbaad764c99" ns2:_="" ns3:_="">
     <xsd:import namespace="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
@@ -2931,34 +2532,82 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
-    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
+      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
+      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
+    </_dlc_DocIdUrl>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70706F67-F4D0-436B-9C39-1388BCD46E53}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2975,4 +2624,31 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
+    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
#95: extending Party edit to all admin users.
</commit_message>
<xml_diff>
--- a/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
+++ b/ckan_batch/src/ckan_batch/reader/templates/PIDINST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Drive_D\projects\avre\apps\PIDINST\AuScope-instrument-registry\ckan_batch\src\ckan_batch\reader\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8534A0A-54AC-4895-9665-B63F2F733C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{832795B8-7747-45CF-B9D7-8721B256E704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -930,6 +930,66 @@
     <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -939,15 +999,9 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -956,60 +1010,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1259,7 +1259,7 @@
     <col min="34" max="34" width="20" customWidth="1"/>
     <col min="35" max="37" width="18" customWidth="1"/>
     <col min="38" max="38" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="10.85546875" customWidth="1"/>
     <col min="40" max="43" width="10.28515625" customWidth="1"/>
     <col min="44" max="44" width="10" customWidth="1"/>
     <col min="45" max="45" width="46.28515625" customWidth="1"/>
@@ -1276,120 +1276,120 @@
       <c r="B1" s="6"/>
     </row>
     <row r="2" spans="1:49" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="26"/>
-      <c r="T2" s="26"/>
-      <c r="U2" s="26"/>
-      <c r="V2" s="26"/>
-      <c r="W2" s="26"/>
-      <c r="X2" s="26"/>
-      <c r="Y2" s="26"/>
-      <c r="Z2" s="26"/>
-      <c r="AA2" s="26"/>
-      <c r="AB2" s="26"/>
-      <c r="AC2" s="26"/>
-      <c r="AD2" s="31" t="s">
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="T2" s="17"/>
+      <c r="U2" s="17"/>
+      <c r="V2" s="17"/>
+      <c r="W2" s="17"/>
+      <c r="X2" s="17"/>
+      <c r="Y2" s="17"/>
+      <c r="Z2" s="17"/>
+      <c r="AA2" s="17"/>
+      <c r="AB2" s="17"/>
+      <c r="AC2" s="17"/>
+      <c r="AD2" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="AE2" s="31"/>
-      <c r="AF2" s="31"/>
-      <c r="AG2" s="31"/>
-      <c r="AH2" s="31"/>
-      <c r="AI2" s="31"/>
-      <c r="AJ2" s="31"/>
-      <c r="AK2" s="31"/>
-      <c r="AL2" s="31"/>
-      <c r="AM2" s="31"/>
-      <c r="AN2" s="31"/>
-      <c r="AO2" s="31"/>
-      <c r="AP2" s="31"/>
-      <c r="AQ2" s="31"/>
-      <c r="AR2" s="31"/>
-      <c r="AS2" s="31" t="s">
+      <c r="AE2" s="22"/>
+      <c r="AF2" s="22"/>
+      <c r="AG2" s="22"/>
+      <c r="AH2" s="22"/>
+      <c r="AI2" s="22"/>
+      <c r="AJ2" s="22"/>
+      <c r="AK2" s="22"/>
+      <c r="AL2" s="22"/>
+      <c r="AM2" s="22"/>
+      <c r="AN2" s="22"/>
+      <c r="AO2" s="22"/>
+      <c r="AP2" s="22"/>
+      <c r="AQ2" s="22"/>
+      <c r="AR2" s="22"/>
+      <c r="AS2" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="AT2" s="31"/>
-      <c r="AU2" s="31"/>
-      <c r="AV2" s="31"/>
-      <c r="AW2" s="31"/>
+      <c r="AT2" s="22"/>
+      <c r="AU2" s="22"/>
+      <c r="AV2" s="22"/>
+      <c r="AW2" s="22"/>
     </row>
     <row r="3" spans="1:49" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="42"/>
-      <c r="J3" s="42"/>
-      <c r="K3" s="43"/>
-      <c r="L3" s="38" t="s">
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="31" t="s">
         <v>126</v>
       </c>
-      <c r="M3" s="39"/>
-      <c r="N3" s="39"/>
-      <c r="O3" s="39"/>
-      <c r="P3" s="39"/>
-      <c r="Q3" s="39"/>
-      <c r="R3" s="39"/>
-      <c r="S3" s="39"/>
-      <c r="T3" s="39"/>
-      <c r="U3" s="39"/>
-      <c r="V3" s="39"/>
-      <c r="W3" s="39"/>
-      <c r="X3" s="39"/>
-      <c r="Y3" s="39"/>
-      <c r="Z3" s="39"/>
-      <c r="AA3" s="39"/>
-      <c r="AB3" s="39"/>
-      <c r="AC3" s="40"/>
-      <c r="AD3" s="17" t="s">
+      <c r="M3" s="32"/>
+      <c r="N3" s="32"/>
+      <c r="O3" s="32"/>
+      <c r="P3" s="32"/>
+      <c r="Q3" s="32"/>
+      <c r="R3" s="32"/>
+      <c r="S3" s="32"/>
+      <c r="T3" s="32"/>
+      <c r="U3" s="32"/>
+      <c r="V3" s="32"/>
+      <c r="W3" s="32"/>
+      <c r="X3" s="32"/>
+      <c r="Y3" s="32"/>
+      <c r="Z3" s="32"/>
+      <c r="AA3" s="32"/>
+      <c r="AB3" s="32"/>
+      <c r="AC3" s="33"/>
+      <c r="AD3" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="AE3" s="18"/>
-      <c r="AF3" s="18"/>
-      <c r="AG3" s="18"/>
-      <c r="AH3" s="18"/>
-      <c r="AI3" s="18"/>
-      <c r="AJ3" s="18"/>
-      <c r="AK3" s="18"/>
-      <c r="AL3" s="18"/>
-      <c r="AM3" s="18"/>
-      <c r="AN3" s="18"/>
-      <c r="AO3" s="18"/>
-      <c r="AP3" s="18"/>
-      <c r="AQ3" s="18"/>
-      <c r="AR3" s="19"/>
-      <c r="AS3" s="29" t="s">
+      <c r="AE3" s="38"/>
+      <c r="AF3" s="38"/>
+      <c r="AG3" s="38"/>
+      <c r="AH3" s="38"/>
+      <c r="AI3" s="38"/>
+      <c r="AJ3" s="38"/>
+      <c r="AK3" s="38"/>
+      <c r="AL3" s="38"/>
+      <c r="AM3" s="38"/>
+      <c r="AN3" s="38"/>
+      <c r="AO3" s="38"/>
+      <c r="AP3" s="38"/>
+      <c r="AQ3" s="38"/>
+      <c r="AR3" s="39"/>
+      <c r="AS3" s="20" t="s">
         <v>132</v>
       </c>
-      <c r="AT3" s="30"/>
-      <c r="AU3" s="30"/>
-      <c r="AV3" s="30"/>
-      <c r="AW3" s="30"/>
+      <c r="AT3" s="21"/>
+      <c r="AU3" s="21"/>
+      <c r="AV3" s="21"/>
+      <c r="AW3" s="21"/>
     </row>
     <row r="4" spans="1:49" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
@@ -1405,74 +1405,74 @@
       <c r="E4" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="F4" s="32" t="s">
+      <c r="F4" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="G4" s="33"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="32" t="s">
+      <c r="G4" s="24"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="J4" s="33"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="20" t="s">
+      <c r="J4" s="24"/>
+      <c r="K4" s="25"/>
+      <c r="L4" s="26" t="s">
         <v>110</v>
       </c>
-      <c r="M4" s="22"/>
-      <c r="N4" s="20" t="s">
+      <c r="M4" s="27"/>
+      <c r="N4" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="O4" s="21"/>
-      <c r="P4" s="20" t="s">
+      <c r="O4" s="40"/>
+      <c r="P4" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="23" t="s">
+      <c r="Q4" s="27"/>
+      <c r="R4" s="41" t="s">
         <v>172</v>
       </c>
-      <c r="S4" s="24"/>
-      <c r="T4" s="24"/>
-      <c r="U4" s="24"/>
-      <c r="V4" s="25"/>
-      <c r="W4" s="20" t="s">
+      <c r="S4" s="42"/>
+      <c r="T4" s="42"/>
+      <c r="U4" s="42"/>
+      <c r="V4" s="43"/>
+      <c r="W4" s="26" t="s">
         <v>173</v>
       </c>
-      <c r="X4" s="22"/>
-      <c r="Y4" s="22"/>
-      <c r="Z4" s="22"/>
-      <c r="AA4" s="20" t="s">
+      <c r="X4" s="27"/>
+      <c r="Y4" s="27"/>
+      <c r="Z4" s="27"/>
+      <c r="AA4" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="AB4" s="22"/>
-      <c r="AC4" s="21"/>
-      <c r="AD4" s="35" t="s">
+      <c r="AB4" s="27"/>
+      <c r="AC4" s="40"/>
+      <c r="AD4" s="28" t="s">
         <v>125</v>
       </c>
-      <c r="AE4" s="36"/>
-      <c r="AF4" s="36"/>
-      <c r="AG4" s="37"/>
-      <c r="AH4" s="35" t="s">
+      <c r="AE4" s="29"/>
+      <c r="AF4" s="29"/>
+      <c r="AG4" s="30"/>
+      <c r="AH4" s="28" t="s">
         <v>118</v>
       </c>
-      <c r="AI4" s="37"/>
-      <c r="AJ4" s="35" t="s">
+      <c r="AI4" s="30"/>
+      <c r="AJ4" s="28" t="s">
         <v>119</v>
       </c>
-      <c r="AK4" s="36"/>
-      <c r="AL4" s="36"/>
-      <c r="AM4" s="36"/>
-      <c r="AN4" s="36"/>
-      <c r="AO4" s="36"/>
-      <c r="AP4" s="36"/>
-      <c r="AQ4" s="36"/>
-      <c r="AR4" s="37"/>
-      <c r="AS4" s="27" t="s">
+      <c r="AK4" s="29"/>
+      <c r="AL4" s="29"/>
+      <c r="AM4" s="29"/>
+      <c r="AN4" s="29"/>
+      <c r="AO4" s="29"/>
+      <c r="AP4" s="29"/>
+      <c r="AQ4" s="29"/>
+      <c r="AR4" s="30"/>
+      <c r="AS4" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="AT4" s="28"/>
-      <c r="AU4" s="28"/>
-      <c r="AV4" s="28"/>
-      <c r="AW4" s="28"/>
+      <c r="AT4" s="19"/>
+      <c r="AU4" s="19"/>
+      <c r="AV4" s="19"/>
+      <c r="AW4" s="19"/>
     </row>
     <row r="5" spans="1:49" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -1587,22 +1587,22 @@
         <v>160</v>
       </c>
       <c r="AL5" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="AM5" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="AM5" s="1" t="s">
-        <v>96</v>
-      </c>
       <c r="AN5" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="AO5" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="AO5" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="AP5" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="AQ5" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="AQ5" s="1" t="s">
-        <v>168</v>
       </c>
       <c r="AR5" s="1" t="s">
         <v>19</v>
@@ -1742,16 +1742,16 @@
         <v>155</v>
       </c>
       <c r="AN6" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="AO6" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="AO6" s="2" t="s">
-        <v>157</v>
-      </c>
       <c r="AP6" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="AQ6" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="AQ6" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="AR6" s="2" t="s">
         <v>44</v>
@@ -1771,6 +1771,9 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="R4:V4"/>
+    <mergeCell ref="W4:Z4"/>
+    <mergeCell ref="AA4:AC4"/>
     <mergeCell ref="A2:AC2"/>
     <mergeCell ref="AS4:AW4"/>
     <mergeCell ref="AS3:AW3"/>
@@ -1787,9 +1790,6 @@
     <mergeCell ref="AD3:AR3"/>
     <mergeCell ref="N4:O4"/>
     <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="R4:V4"/>
-    <mergeCell ref="W4:Z4"/>
-    <mergeCell ref="AA4:AC4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
@@ -2271,6 +2271,81 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
+      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
+      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
+    </_dlc_DocIdUrl>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C458252014B43B48B36D6FD06F31079C" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8411b2fcd13e9c262f801c2de01d8359">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9357ce84-a672-4584-8ddb-e5b553dfe263" xmlns:ns3="f66f598c-5a54-48fa-b12a-3e2e658c8d92" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7559adb2811d00dbbd5f4bbaad764c99" ns2:_="" ns3:_="">
     <xsd:import namespace="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
@@ -2532,82 +2607,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
+    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">6KAJUDXX5TY3-1158213377-2347</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263">
-      <Url>https://csiroau.sharepoint.com/sites/AuScopePortalRefresh/_layouts/15/DocIdRedir.aspx?ID=6KAJUDXX5TY3-1158213377-2347</Url>
-      <Description>6KAJUDXX5TY3-1158213377-2347</Description>
-    </_dlc_DocIdUrl>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f66f598c-5a54-48fa-b12a-3e2e658c8d92">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9357ce84-a672-4584-8ddb-e5b553dfe263" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70706F67-F4D0-436B-9C39-1388BCD46E53}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2624,31 +2651,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FB246EF-5385-459E-BC46-E2D2C91CAB60}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B91B4E20-BE34-4CB5-9F97-891AD3D92955}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67E57F81-9D8B-47B3-8107-9966928F030D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
-    <ds:schemaRef ds:uri="f66f598c-5a54-48fa-b12a-3e2e658c8d92"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>